<commit_message>
Updating the encounter tracking sheet
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\petrona\pokefirered-expansion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9E96127F-8262-4FDA-9FE2-0F13D02C689D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9B265D-6796-458D-81EA-9F7532223980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28905" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="429">
   <si>
     <t>Species</t>
   </si>
@@ -1251,6 +1251,78 @@
   </si>
   <si>
     <t>ROUTE5</t>
+  </si>
+  <si>
+    <t>MT_EMBER_EXTERIOR</t>
+  </si>
+  <si>
+    <t>CRITTER_CAVE Fishing</t>
+  </si>
+  <si>
+    <t>MT_MOON_B2F</t>
+  </si>
+  <si>
+    <t>MT_EMBER_RUBY_PATH_B2F_STAIRS Rock Smash</t>
+  </si>
+  <si>
+    <t>SAFARI_ZONE_EAST Water</t>
+  </si>
+  <si>
+    <t>CERULEAN_CAVE_B1F Water</t>
+  </si>
+  <si>
+    <t>POKEMON_TOWER_7F</t>
+  </si>
+  <si>
+    <t>VICTORY_ROAD_3F</t>
+  </si>
+  <si>
+    <t>ROUTE25</t>
+  </si>
+  <si>
+    <t>FOUR_ISLAND_ICEFALL_CAVE_ENTRANCE</t>
+  </si>
+  <si>
+    <t>ROCK_TUNNEL_2F</t>
+  </si>
+  <si>
+    <t>SAFARI_ZONE_CENTER</t>
+  </si>
+  <si>
+    <t>ROUTE4 Fishing</t>
+  </si>
+  <si>
+    <t>ROUTE19 Water</t>
+  </si>
+  <si>
+    <t>ROUTE18</t>
+  </si>
+  <si>
+    <t>MT_EMBER_RUBY_PATH_B1F</t>
+  </si>
+  <si>
+    <t>SAFARI_ZONE_CENTER Fishing</t>
+  </si>
+  <si>
+    <t>ROUTE20 Fishing</t>
+  </si>
+  <si>
+    <t>SSANNE_EXTERIOR Water</t>
+  </si>
+  <si>
+    <t>SEAFOAM_ISLANDS_B4F</t>
+  </si>
+  <si>
+    <t>MT_EMBER_SUMMIT_PATH_3F</t>
+  </si>
+  <si>
+    <t>ROUTE1 Water</t>
+  </si>
+  <si>
+    <t>ROUTE10 Fishing</t>
+  </si>
+  <si>
+    <t>FOUR_ISLAND_ICEFALL_CAVE_BACK Fishing</t>
   </si>
 </sst>
 </file>
@@ -1648,13 +1720,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
   <dimension ref="A1:B335"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7265625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1662,7 +1734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1670,7 +1742,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1678,7 +1750,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1686,7 +1758,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -1694,7 +1766,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1702,7 +1774,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -1710,7 +1782,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1718,7 +1790,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1726,7 +1798,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1734,7 +1806,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1742,7 +1814,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -1750,7 +1822,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -1758,7 +1830,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -1766,7 +1838,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -1774,7 +1846,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1782,7 +1854,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -1790,7 +1862,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
@@ -1798,7 +1870,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
@@ -1806,7 +1878,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -1814,7 +1886,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
@@ -1822,7 +1894,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -1830,7 +1902,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -1838,7 +1910,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>24</v>
       </c>
@@ -1846,7 +1918,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -1854,7 +1926,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
@@ -1862,7 +1934,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -1870,7 +1942,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>28</v>
       </c>
@@ -1878,7 +1950,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>29</v>
       </c>
@@ -1886,7 +1958,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
@@ -1894,7 +1966,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
@@ -1902,7 +1974,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
@@ -1910,7 +1982,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
@@ -1918,7 +1990,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
@@ -1926,7 +1998,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>35</v>
       </c>
@@ -1934,7 +2006,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>36</v>
       </c>
@@ -1942,7 +2014,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>37</v>
       </c>
@@ -1950,7 +2022,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
@@ -1958,7 +2030,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>39</v>
       </c>
@@ -1966,7 +2038,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>40</v>
       </c>
@@ -1974,7 +2046,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>41</v>
       </c>
@@ -1982,7 +2054,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>42</v>
       </c>
@@ -1990,7 +2062,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>43</v>
       </c>
@@ -1998,7 +2070,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>44</v>
       </c>
@@ -2006,7 +2078,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>45</v>
       </c>
@@ -2014,7 +2086,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>46</v>
       </c>
@@ -2022,7 +2094,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>47</v>
       </c>
@@ -2030,7 +2102,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
@@ -2038,7 +2110,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>49</v>
       </c>
@@ -2046,7 +2118,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>50</v>
       </c>
@@ -2054,7 +2126,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="3" t="s">
         <v>51</v>
       </c>
@@ -2062,7 +2134,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>52</v>
       </c>
@@ -2070,7 +2142,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
@@ -2078,7 +2150,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>54</v>
       </c>
@@ -2086,7 +2158,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="3" t="s">
         <v>55</v>
       </c>
@@ -2094,7 +2166,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>56</v>
       </c>
@@ -2102,7 +2174,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>57</v>
       </c>
@@ -2110,7 +2182,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>58</v>
       </c>
@@ -2118,7 +2190,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
@@ -2126,7 +2198,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>60</v>
       </c>
@@ -2134,7 +2206,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
@@ -2142,7 +2214,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>62</v>
       </c>
@@ -2150,7 +2222,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>63</v>
       </c>
@@ -2158,7 +2230,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>64</v>
       </c>
@@ -2166,7 +2238,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -2174,7 +2246,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
@@ -2182,7 +2254,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
@@ -2190,7 +2262,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" s="3" t="s">
         <v>68</v>
       </c>
@@ -2198,7 +2270,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
@@ -2206,7 +2278,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
@@ -2214,7 +2286,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
@@ -2222,7 +2294,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
@@ -2230,7 +2302,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
@@ -2238,7 +2310,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>74</v>
       </c>
@@ -2246,7 +2318,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
@@ -2254,7 +2326,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
@@ -2262,7 +2334,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
@@ -2270,7 +2342,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
@@ -2278,7 +2350,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
@@ -2286,7 +2358,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
@@ -2294,7 +2366,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
@@ -2302,7 +2374,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>82</v>
       </c>
@@ -2310,7 +2382,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
@@ -2318,7 +2390,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
@@ -2326,7 +2398,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>85</v>
       </c>
@@ -2334,7 +2406,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
@@ -2342,7 +2414,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
@@ -2350,7 +2422,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" s="3" t="s">
         <v>88</v>
       </c>
@@ -2358,7 +2430,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>89</v>
       </c>
@@ -2366,7 +2438,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>90</v>
       </c>
@@ -2374,7 +2446,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>91</v>
       </c>
@@ -2382,7 +2454,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>92</v>
       </c>
@@ -2390,7 +2462,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>93</v>
       </c>
@@ -2398,7 +2470,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>94</v>
       </c>
@@ -2406,7 +2478,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>95</v>
       </c>
@@ -2414,7 +2486,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
@@ -2422,7 +2494,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>97</v>
       </c>
@@ -2430,7 +2502,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>98</v>
       </c>
@@ -2438,7 +2510,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>99</v>
       </c>
@@ -2446,7 +2518,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>100</v>
       </c>
@@ -2454,7 +2526,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>101</v>
       </c>
@@ -2462,7 +2534,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>102</v>
       </c>
@@ -2470,7 +2542,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>103</v>
       </c>
@@ -2478,7 +2550,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>104</v>
       </c>
@@ -2486,7 +2558,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>105</v>
       </c>
@@ -2494,7 +2566,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>106</v>
       </c>
@@ -2502,7 +2574,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>107</v>
       </c>
@@ -2510,7 +2582,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>108</v>
       </c>
@@ -2518,7 +2590,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>109</v>
       </c>
@@ -2526,7 +2598,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" s="3" t="s">
         <v>110</v>
       </c>
@@ -2534,7 +2606,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>111</v>
       </c>
@@ -2542,7 +2614,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>112</v>
       </c>
@@ -2550,7 +2622,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>113</v>
       </c>
@@ -2558,7 +2630,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>114</v>
       </c>
@@ -2566,7 +2638,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>115</v>
       </c>
@@ -2574,7 +2646,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>116</v>
       </c>
@@ -2582,7 +2654,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>117</v>
       </c>
@@ -2590,7 +2662,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>118</v>
       </c>
@@ -2598,7 +2670,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>119</v>
       </c>
@@ -2606,7 +2678,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>120</v>
       </c>
@@ -2614,7 +2686,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>121</v>
       </c>
@@ -2622,7 +2694,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>122</v>
       </c>
@@ -2630,7 +2702,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>123</v>
       </c>
@@ -2638,7 +2710,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>124</v>
       </c>
@@ -2646,7 +2718,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>125</v>
       </c>
@@ -2654,7 +2726,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>126</v>
       </c>
@@ -2662,7 +2734,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>127</v>
       </c>
@@ -2670,7 +2742,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A128" s="3" t="s">
         <v>128</v>
       </c>
@@ -2678,7 +2750,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>129</v>
       </c>
@@ -2686,7 +2758,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>130</v>
       </c>
@@ -2694,7 +2766,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>131</v>
       </c>
@@ -2702,7 +2774,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>132</v>
       </c>
@@ -2710,7 +2782,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>133</v>
       </c>
@@ -2718,7 +2790,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>134</v>
       </c>
@@ -2726,7 +2798,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>135</v>
       </c>
@@ -2734,7 +2806,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>136</v>
       </c>
@@ -2742,7 +2814,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>137</v>
       </c>
@@ -2750,7 +2822,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>138</v>
       </c>
@@ -2758,7 +2830,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>139</v>
       </c>
@@ -2766,7 +2838,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>140</v>
       </c>
@@ -2774,7 +2846,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>141</v>
       </c>
@@ -2782,7 +2854,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>142</v>
       </c>
@@ -2790,7 +2862,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>143</v>
       </c>
@@ -2798,7 +2870,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>144</v>
       </c>
@@ -2806,7 +2878,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
@@ -2814,7 +2886,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>146</v>
       </c>
@@ -2822,7 +2894,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>147</v>
       </c>
@@ -2830,7 +2902,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>148</v>
       </c>
@@ -2838,7 +2910,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>149</v>
       </c>
@@ -2846,7 +2918,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>150</v>
       </c>
@@ -2854,7 +2926,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>151</v>
       </c>
@@ -2862,7 +2934,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>152</v>
       </c>
@@ -2870,7 +2942,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>153</v>
       </c>
@@ -2878,7 +2950,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>154</v>
       </c>
@@ -2886,7 +2958,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>155</v>
       </c>
@@ -2894,7 +2966,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>156</v>
       </c>
@@ -2902,7 +2974,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>157</v>
       </c>
@@ -2910,7 +2982,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>158</v>
       </c>
@@ -2918,7 +2990,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>159</v>
       </c>
@@ -2926,7 +2998,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>160</v>
       </c>
@@ -2934,7 +3006,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>161</v>
       </c>
@@ -2942,7 +3014,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>162</v>
       </c>
@@ -2950,7 +3022,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>163</v>
       </c>
@@ -2958,7 +3030,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>164</v>
       </c>
@@ -2966,7 +3038,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>165</v>
       </c>
@@ -2974,7 +3046,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>166</v>
       </c>
@@ -2982,7 +3054,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>167</v>
       </c>
@@ -2990,7 +3062,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>168</v>
       </c>
@@ -2998,7 +3070,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>169</v>
       </c>
@@ -3006,7 +3078,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>170</v>
       </c>
@@ -3014,7 +3086,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>171</v>
       </c>
@@ -3022,822 +3094,1159 @@
         <v>337</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B172" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B173" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B174" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B175" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B176" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B177" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B178" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B179" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B180" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B181" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B182" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B183" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B184" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B185" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B186" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B187" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B188" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B189" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B190" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B191" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A193" s="1" t="s">
+      <c r="B192" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A193" s="3" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B193" s="4"/>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B194" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B195" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B196" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B197" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B198" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B199" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B200" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B201" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>202</v>
       </c>
-    </row>
-    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B202" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B203" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B204" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B205" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B206" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B207" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B208" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B209" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B210" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B211" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B212" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B213" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B214" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B215" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B216" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B217" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B218" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B219" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B220" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B221" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B222" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B223" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>224</v>
       </c>
-    </row>
-    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B224" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B225" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B226" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B227" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>228</v>
       </c>
-    </row>
-    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B228" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B229" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B230" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B231" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B232" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B233" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B234" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B235" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B236" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B237" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>238</v>
       </c>
-    </row>
-    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B238" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B239" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B240" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B241" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B242" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B243" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B244" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B245" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B246" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B247" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B248" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B249" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B250" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B251" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>252</v>
       </c>
-    </row>
-    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B252" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B253" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B254" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B255" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B256" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B257" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B258" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B259" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>260</v>
       </c>
-    </row>
-    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B260" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B261" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B262" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B263" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B264" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B265" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B266" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B267" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B268" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B269" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B270" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B271" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B272" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B273" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B274" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B275" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B276" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A278" s="1" t="s">
+      <c r="B277" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A278" s="3" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B278" s="4" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B279" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B280" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B281" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B282" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B283" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>284</v>
       </c>
-    </row>
-    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B284" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>298</v>
       </c>
     </row>
-    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>306</v>
       </c>
     </row>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>307</v>
       </c>
     </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>308</v>
       </c>
     </row>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>309</v>
       </c>
     </row>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>310</v>
       </c>
     </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>314</v>
       </c>
     </row>
-    <row r="315" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="316" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>316</v>
       </c>
     </row>
-    <row r="317" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>317</v>
       </c>
     </row>
-    <row r="318" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>318</v>
       </c>
     </row>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>321</v>
       </c>
     </row>
-    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>327</v>
       </c>
     </row>
-    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>329</v>
       </c>
     </row>
-    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>331</v>
       </c>
     </row>
-    <row r="332" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="333" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="334" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>334</v>
       </c>
     </row>
-    <row r="335" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>335</v>
       </c>

</xml_diff>

<commit_message>
Updating encounter tracking sheet
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9B265D-6796-458D-81EA-9F7532223980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8903FE-424D-49E2-83E6-7D4149BD10C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1235" uniqueCount="429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="435">
   <si>
     <t>Species</t>
   </si>
@@ -1283,6 +1283,9 @@
     <t>FOUR_ISLAND_ICEFALL_CAVE_ENTRANCE</t>
   </si>
   <si>
+    <t>POKEMON_TOWER_6F</t>
+  </si>
+  <si>
     <t>ROCK_TUNNEL_2F</t>
   </si>
   <si>
@@ -1323,6 +1326,21 @@
   </si>
   <si>
     <t>FOUR_ISLAND_ICEFALL_CAVE_BACK Fishing</t>
+  </si>
+  <si>
+    <t>CERULEAN_CAVE_1F Water</t>
+  </si>
+  <si>
+    <t>ROUTE1 Fishing</t>
+  </si>
+  <si>
+    <t>Static Encounter</t>
+  </si>
+  <si>
+    <t>Route4</t>
+  </si>
+  <si>
+    <t>Roamer</t>
   </si>
 </sst>
 </file>
@@ -3417,7 +3435,7 @@
         <v>212</v>
       </c>
       <c r="B212" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="213" spans="1:2" x14ac:dyDescent="0.35">
@@ -3521,7 +3539,7 @@
         <v>225</v>
       </c>
       <c r="B225" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
     </row>
     <row r="226" spans="1:2" x14ac:dyDescent="0.35">
@@ -3529,7 +3547,7 @@
         <v>226</v>
       </c>
       <c r="B226" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="227" spans="1:2" x14ac:dyDescent="0.35">
@@ -3537,7 +3555,7 @@
         <v>227</v>
       </c>
       <c r="B227" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="228" spans="1:2" x14ac:dyDescent="0.35">
@@ -3665,7 +3683,7 @@
         <v>243</v>
       </c>
       <c r="B243" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="244" spans="1:2" x14ac:dyDescent="0.35">
@@ -3673,7 +3691,7 @@
         <v>244</v>
       </c>
       <c r="B244" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="245" spans="1:2" x14ac:dyDescent="0.35">
@@ -3721,7 +3739,7 @@
         <v>250</v>
       </c>
       <c r="B250" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="251" spans="1:2" x14ac:dyDescent="0.35">
@@ -3777,7 +3795,7 @@
         <v>257</v>
       </c>
       <c r="B257" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="258" spans="1:2" x14ac:dyDescent="0.35">
@@ -3801,7 +3819,7 @@
         <v>260</v>
       </c>
       <c r="B260" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="261" spans="1:2" x14ac:dyDescent="0.35">
@@ -3809,7 +3827,7 @@
         <v>261</v>
       </c>
       <c r="B261" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="262" spans="1:2" x14ac:dyDescent="0.35">
@@ -3873,7 +3891,7 @@
         <v>269</v>
       </c>
       <c r="B269" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="270" spans="1:2" x14ac:dyDescent="0.35">
@@ -3881,7 +3899,7 @@
         <v>270</v>
       </c>
       <c r="B270" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="271" spans="1:2" x14ac:dyDescent="0.35">
@@ -3929,7 +3947,7 @@
         <v>276</v>
       </c>
       <c r="B276" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="277" spans="1:2" x14ac:dyDescent="0.35">
@@ -3945,7 +3963,7 @@
         <v>278</v>
       </c>
       <c r="B278" s="4" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="279" spans="1:2" x14ac:dyDescent="0.35">
@@ -3953,7 +3971,7 @@
         <v>279</v>
       </c>
       <c r="B279" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="280" spans="1:2" x14ac:dyDescent="0.35">
@@ -3961,7 +3979,7 @@
         <v>280</v>
       </c>
       <c r="B280" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="281" spans="1:2" x14ac:dyDescent="0.35">
@@ -3969,7 +3987,7 @@
         <v>281</v>
       </c>
       <c r="B281" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="282" spans="1:2" x14ac:dyDescent="0.35">
@@ -3985,7 +4003,7 @@
         <v>283</v>
       </c>
       <c r="B283" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="284" spans="1:2" x14ac:dyDescent="0.35">
@@ -3993,262 +4011,413 @@
         <v>284</v>
       </c>
       <c r="B284" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
     </row>
     <row r="285" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A285" s="1" t="s">
+      <c r="A285" s="3" t="s">
         <v>285</v>
       </c>
+      <c r="B285" s="4"/>
     </row>
     <row r="286" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>286</v>
       </c>
+      <c r="B286" t="s">
+        <v>374</v>
+      </c>
     </row>
     <row r="287" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>287</v>
       </c>
+      <c r="B287" t="s">
+        <v>407</v>
+      </c>
     </row>
     <row r="288" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="289" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B288" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="290" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B289" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="291" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B290" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="292" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B291" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>292</v>
       </c>
-    </row>
-    <row r="293" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B292" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="294" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B293" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="295" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B294" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="296" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B295" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="297" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B296" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="298" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B297" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>298</v>
       </c>
-    </row>
-    <row r="299" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B298" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="300" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B299" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="301" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B300" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="302" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B301" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>302</v>
       </c>
-    </row>
-    <row r="303" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B302" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="304" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B303" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B304" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="306" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B305" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>306</v>
       </c>
-    </row>
-    <row r="307" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B306" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="308" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B307" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>308</v>
       </c>
-    </row>
-    <row r="309" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B308" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="310" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B309" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>310</v>
       </c>
-    </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B310" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="312" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B311" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>312</v>
       </c>
-    </row>
-    <row r="313" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B312" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="314" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B313" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="315" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B314" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="316" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B315" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>316</v>
       </c>
-    </row>
-    <row r="317" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B316" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="318" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B317" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>318</v>
       </c>
-    </row>
-    <row r="319" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B318" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="320" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B319" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>320</v>
       </c>
-    </row>
-    <row r="321" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B320" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="322" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B321" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B322" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="324" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B323" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>324</v>
       </c>
-    </row>
-    <row r="325" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B324" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="326" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B325" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="327" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B326" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="328" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B327" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="329" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B328" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="330" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B329" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>330</v>
       </c>
-    </row>
-    <row r="331" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B330" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="332" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B331" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>332</v>
       </c>
-    </row>
-    <row r="333" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B332" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="334" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B333" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="335" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="B334" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>335</v>
+      </c>
+      <c r="B335" t="s">
+        <v>432</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes to encounters according to tracker
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\petrona\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F8903FE-424D-49E2-83E6-7D4149BD10C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B66B2C-232D-4A8A-8D32-A1C28108C6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
+    <workbookView xWindow="-28890" yWindow="2800" windowWidth="9780" windowHeight="11370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="433">
   <si>
     <t>Species</t>
   </si>
@@ -1127,9 +1127,6 @@
     <t>ROUTE22 Fishing</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>CERULEAN_CAVE_B1F</t>
   </si>
   <si>
@@ -1197,9 +1194,6 @@
   </si>
   <si>
     <t>SEAFOAM_ISLANDS_1F</t>
-  </si>
-  <si>
-    <t>MT_EMBER_SUMMIT_PATH_2F Rock Smash</t>
   </si>
   <si>
     <t>SEAFOAM_ISLANDS_B2F</t>
@@ -1393,7 +1387,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1403,6 +1397,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1738,13 +1736,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
   <dimension ref="A1:B335"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1752,7 +1750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1760,7 +1758,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1768,7 +1766,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1776,7 +1774,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -1784,7 +1782,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1792,7 +1790,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -1800,7 +1798,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1808,7 +1806,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1816,7 +1814,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1824,7 +1822,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1832,7 +1830,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -1840,7 +1838,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -1848,7 +1846,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -1856,7 +1854,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -1864,7 +1862,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -1872,7 +1870,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -1880,7 +1878,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
@@ -1888,7 +1886,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
@@ -1896,7 +1894,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -1904,7 +1902,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
@@ -1912,7 +1910,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -1920,7 +1918,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -1928,7 +1926,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>24</v>
       </c>
@@ -1936,7 +1934,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -1944,7 +1942,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
@@ -1952,7 +1950,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -1960,7 +1958,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>28</v>
       </c>
@@ -1968,15 +1966,15 @@
         <v>348</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B29" s="6" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
@@ -1984,7 +1982,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
@@ -1992,7 +1990,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
@@ -2000,7 +1998,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
@@ -2008,7 +2006,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
@@ -2016,7 +2014,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>35</v>
       </c>
@@ -2024,7 +2022,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>36</v>
       </c>
@@ -2032,7 +2030,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>37</v>
       </c>
@@ -2040,7 +2038,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
@@ -2048,7 +2046,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>39</v>
       </c>
@@ -2056,7 +2054,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>40</v>
       </c>
@@ -2064,7 +2062,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>41</v>
       </c>
@@ -2072,7 +2070,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>42</v>
       </c>
@@ -2080,7 +2078,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>43</v>
       </c>
@@ -2088,7 +2086,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>44</v>
       </c>
@@ -2096,7 +2094,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>45</v>
       </c>
@@ -2104,7 +2102,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>46</v>
       </c>
@@ -2112,7 +2110,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>47</v>
       </c>
@@ -2120,7 +2118,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
@@ -2128,7 +2126,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>49</v>
       </c>
@@ -2136,7 +2134,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>50</v>
       </c>
@@ -2144,23 +2142,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A51" s="3" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B51" s="6" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B52" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
@@ -2168,7 +2166,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>54</v>
       </c>
@@ -2176,23 +2174,23 @@
         <v>351</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A55" s="3" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B55" s="6" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B56" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>57</v>
       </c>
@@ -2200,15 +2198,15 @@
         <v>339</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B58" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
@@ -2216,23 +2214,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B61" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>62</v>
       </c>
@@ -2240,15 +2238,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>64</v>
       </c>
@@ -2256,23 +2254,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
@@ -2280,23 +2278,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A68" s="3" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B68" s="6" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B69" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
@@ -2304,7 +2302,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
@@ -2312,7 +2310,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
@@ -2320,55 +2318,55 @@
         <v>336</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B73" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B74" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B75" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B77" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
@@ -2376,23 +2374,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B80" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>82</v>
       </c>
@@ -2400,7 +2398,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
@@ -2408,7 +2406,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
@@ -2416,7 +2414,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>85</v>
       </c>
@@ -2424,31 +2422,31 @@
         <v>337</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B87" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A88" s="3" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B88" s="4" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B88" s="6" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>89</v>
       </c>
@@ -2456,15 +2454,15 @@
         <v>355</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B90" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>91</v>
       </c>
@@ -2472,7 +2470,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>92</v>
       </c>
@@ -2480,15 +2478,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B93" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>94</v>
       </c>
@@ -2496,47 +2494,47 @@
         <v>337</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B95" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
       <c r="B96" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>97</v>
       </c>
       <c r="B97" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B98" t="s">
-        <v>382</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B99" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>100</v>
       </c>
@@ -2544,7 +2542,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>101</v>
       </c>
@@ -2552,7 +2550,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>102</v>
       </c>
@@ -2560,7 +2558,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>103</v>
       </c>
@@ -2568,7 +2566,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>104</v>
       </c>
@@ -2576,7 +2574,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>105</v>
       </c>
@@ -2584,7 +2582,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>106</v>
       </c>
@@ -2592,7 +2590,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>107</v>
       </c>
@@ -2600,15 +2598,15 @@
         <v>341</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B108" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>109</v>
       </c>
@@ -2616,23 +2614,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A110" s="3" t="s">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="B110" s="4" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B110" s="6" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B111" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>112</v>
       </c>
@@ -2640,7 +2638,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>113</v>
       </c>
@@ -2648,15 +2646,15 @@
         <v>336</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B114" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>115</v>
       </c>
@@ -2664,7 +2662,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>116</v>
       </c>
@@ -2672,7 +2670,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>117</v>
       </c>
@@ -2680,7 +2678,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>118</v>
       </c>
@@ -2688,7 +2686,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>119</v>
       </c>
@@ -2696,7 +2694,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>120</v>
       </c>
@@ -2704,7 +2702,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>121</v>
       </c>
@@ -2712,7 +2710,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>122</v>
       </c>
@@ -2720,15 +2718,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>123</v>
       </c>
       <c r="B123" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>124</v>
       </c>
@@ -2736,7 +2734,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>125</v>
       </c>
@@ -2744,15 +2742,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>126</v>
       </c>
       <c r="B126" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>127</v>
       </c>
@@ -2760,15 +2758,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A128" s="3" t="s">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B128" s="4" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B128" s="6" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>129</v>
       </c>
@@ -2776,15 +2774,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B130" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>131</v>
       </c>
@@ -2792,15 +2790,15 @@
         <v>340</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B132" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>133</v>
       </c>
@@ -2808,15 +2806,15 @@
         <v>342</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B134" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>135</v>
       </c>
@@ -2824,7 +2822,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>136</v>
       </c>
@@ -2832,31 +2830,31 @@
         <v>337</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B137" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B138" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.35">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>139</v>
       </c>
       <c r="B139" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.35">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>140</v>
       </c>
@@ -2864,7 +2862,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>141</v>
       </c>
@@ -2872,15 +2870,15 @@
         <v>343</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>142</v>
       </c>
       <c r="B142" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.35">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>143</v>
       </c>
@@ -2888,15 +2886,15 @@
         <v>343</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B144" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
@@ -2904,15 +2902,15 @@
         <v>349</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B146" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>147</v>
       </c>
@@ -2920,7 +2918,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>148</v>
       </c>
@@ -2928,15 +2926,15 @@
         <v>343</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B149" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>150</v>
       </c>
@@ -2944,7 +2942,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>151</v>
       </c>
@@ -2952,31 +2950,31 @@
         <v>346</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B152" t="s">
-        <v>386</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B153" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>154</v>
       </c>
       <c r="B154" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>155</v>
       </c>
@@ -2984,7 +2982,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>156</v>
       </c>
@@ -2992,15 +2990,15 @@
         <v>342</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B157" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>158</v>
       </c>
@@ -3008,15 +3006,15 @@
         <v>361</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>159</v>
       </c>
       <c r="B159" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>160</v>
       </c>
@@ -3024,31 +3022,31 @@
         <v>337</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>161</v>
       </c>
       <c r="B161" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B162" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>163</v>
       </c>
       <c r="B163" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>164</v>
       </c>
@@ -3056,15 +3054,15 @@
         <v>346</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>165</v>
       </c>
       <c r="B165" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>166</v>
       </c>
@@ -3072,7 +3070,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>167</v>
       </c>
@@ -3080,31 +3078,31 @@
         <v>341</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>168</v>
       </c>
       <c r="B168" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.35">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>169</v>
       </c>
       <c r="B169" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>170</v>
       </c>
       <c r="B170" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.35">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>171</v>
       </c>
@@ -3112,7 +3110,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>172</v>
       </c>
@@ -3120,15 +3118,15 @@
         <v>343</v>
       </c>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>173</v>
       </c>
       <c r="B173" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.35">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>174</v>
       </c>
@@ -3136,15 +3134,15 @@
         <v>342</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>175</v>
       </c>
       <c r="B175" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.35">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>176</v>
       </c>
@@ -3152,39 +3150,39 @@
         <v>343</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>177</v>
       </c>
       <c r="B177" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>178</v>
       </c>
       <c r="B178" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.35">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>179</v>
       </c>
       <c r="B179" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>180</v>
       </c>
       <c r="B180" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.35">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>181</v>
       </c>
@@ -3192,23 +3190,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>182</v>
       </c>
       <c r="B182" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.35">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>183</v>
       </c>
       <c r="B183" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.35">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>184</v>
       </c>
@@ -3216,15 +3214,15 @@
         <v>339</v>
       </c>
     </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>185</v>
       </c>
       <c r="B185" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>186</v>
       </c>
@@ -3232,15 +3230,15 @@
         <v>342</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>187</v>
       </c>
       <c r="B187" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.35">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>188</v>
       </c>
@@ -3248,15 +3246,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>189</v>
       </c>
       <c r="B189" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.35">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>190</v>
       </c>
@@ -3264,7 +3262,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>191</v>
       </c>
@@ -3272,7 +3270,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>192</v>
       </c>
@@ -3280,21 +3278,21 @@
         <v>359</v>
       </c>
     </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A193" s="3" t="s">
         <v>193</v>
       </c>
       <c r="B193" s="4"/>
     </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>194</v>
       </c>
       <c r="B194" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.35">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>195</v>
       </c>
@@ -3302,15 +3300,15 @@
         <v>349</v>
       </c>
     </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>196</v>
       </c>
       <c r="B196" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.35">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>197</v>
       </c>
@@ -3318,15 +3316,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>198</v>
       </c>
       <c r="B198" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>199</v>
       </c>
@@ -3334,39 +3332,39 @@
         <v>351</v>
       </c>
     </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>200</v>
       </c>
       <c r="B200" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>201</v>
       </c>
       <c r="B201" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>202</v>
       </c>
       <c r="B202" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.35">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>203</v>
       </c>
       <c r="B203" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.35">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>204</v>
       </c>
@@ -3374,39 +3372,39 @@
         <v>337</v>
       </c>
     </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>205</v>
       </c>
       <c r="B205" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.35">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>206</v>
       </c>
       <c r="B206" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>207</v>
       </c>
       <c r="B207" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.35">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>208</v>
       </c>
       <c r="B208" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>209</v>
       </c>
@@ -3414,7 +3412,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>210</v>
       </c>
@@ -3422,39 +3420,39 @@
         <v>337</v>
       </c>
     </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B211" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>212</v>
       </c>
       <c r="B212" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.35">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>213</v>
       </c>
       <c r="B213" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.35">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B214" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>215</v>
       </c>
@@ -3462,15 +3460,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>216</v>
       </c>
       <c r="B216" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.35">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>217</v>
       </c>
@@ -3478,15 +3476,15 @@
         <v>359</v>
       </c>
     </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>218</v>
       </c>
       <c r="B218" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>219</v>
       </c>
@@ -3494,7 +3492,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>220</v>
       </c>
@@ -3502,23 +3500,23 @@
         <v>361</v>
       </c>
     </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>221</v>
       </c>
       <c r="B221" t="s">
-        <v>366</v>
-      </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.35">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A222" s="1" t="s">
         <v>222</v>
       </c>
       <c r="B222" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.35">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A223" s="1" t="s">
         <v>223</v>
       </c>
@@ -3526,39 +3524,39 @@
         <v>360</v>
       </c>
     </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A224" s="1" t="s">
         <v>224</v>
       </c>
       <c r="B224" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.35">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A225" s="1" t="s">
         <v>225</v>
       </c>
       <c r="B225" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.35">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A226" s="1" t="s">
         <v>226</v>
       </c>
       <c r="B226" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.35">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A227" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B227" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.35">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A228" s="1" t="s">
         <v>228</v>
       </c>
@@ -3566,7 +3564,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A229" s="1" t="s">
         <v>229</v>
       </c>
@@ -3574,15 +3572,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A230" s="1" t="s">
         <v>230</v>
       </c>
       <c r="B230" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A231" s="1" t="s">
         <v>231</v>
       </c>
@@ -3590,7 +3588,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A232" s="1" t="s">
         <v>232</v>
       </c>
@@ -3598,15 +3596,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A233" s="1" t="s">
         <v>233</v>
       </c>
       <c r="B233" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A234" s="1" t="s">
         <v>234</v>
       </c>
@@ -3614,7 +3612,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A235" s="1" t="s">
         <v>235</v>
       </c>
@@ -3622,15 +3620,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A236" s="1" t="s">
         <v>236</v>
       </c>
       <c r="B236" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A237" s="1" t="s">
         <v>237</v>
       </c>
@@ -3638,7 +3636,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A238" s="1" t="s">
         <v>238</v>
       </c>
@@ -3646,111 +3644,111 @@
         <v>337</v>
       </c>
     </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A239" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B239" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A240" s="1" t="s">
         <v>240</v>
       </c>
       <c r="B240" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
         <v>241</v>
       </c>
       <c r="B241" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A242" s="1" t="s">
         <v>242</v>
       </c>
       <c r="B242" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.35">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A243" s="1" t="s">
         <v>243</v>
       </c>
       <c r="B243" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.35">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A244" s="1" t="s">
         <v>244</v>
       </c>
       <c r="B244" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.35">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
         <v>245</v>
       </c>
       <c r="B245" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A246" s="1" t="s">
         <v>246</v>
       </c>
       <c r="B246" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A247" s="1" t="s">
         <v>247</v>
       </c>
       <c r="B247" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A248" s="1" t="s">
         <v>248</v>
       </c>
       <c r="B248" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A249" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B249" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A250" s="1" t="s">
         <v>250</v>
       </c>
       <c r="B250" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.35">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A251" s="1" t="s">
         <v>251</v>
       </c>
       <c r="B251" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.35">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A252" s="1" t="s">
         <v>252</v>
       </c>
@@ -3758,15 +3756,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A253" s="1" t="s">
         <v>253</v>
       </c>
       <c r="B253" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A254" s="1" t="s">
         <v>254</v>
       </c>
@@ -3774,7 +3772,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A255" s="1" t="s">
         <v>255</v>
       </c>
@@ -3782,7 +3780,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A256" s="1" t="s">
         <v>256</v>
       </c>
@@ -3790,47 +3788,47 @@
         <v>361</v>
       </c>
     </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A257" s="1" t="s">
         <v>257</v>
       </c>
       <c r="B257" t="s">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.35">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A258" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B258" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A259" s="1" t="s">
         <v>259</v>
       </c>
       <c r="B259" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.35">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A260" s="1" t="s">
         <v>260</v>
       </c>
       <c r="B260" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.35">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A261" s="1" t="s">
         <v>261</v>
       </c>
       <c r="B261" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.35">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A262" s="1" t="s">
         <v>262</v>
       </c>
@@ -3838,15 +3836,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A263" s="1" t="s">
         <v>263</v>
       </c>
       <c r="B263" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.35">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A264" s="1" t="s">
         <v>264</v>
       </c>
@@ -3854,15 +3852,15 @@
         <v>350</v>
       </c>
     </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A265" s="1" t="s">
         <v>265</v>
       </c>
       <c r="B265" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A266" s="1" t="s">
         <v>266</v>
       </c>
@@ -3870,39 +3868,39 @@
         <v>357</v>
       </c>
     </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A267" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B267" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A268" s="1" t="s">
         <v>268</v>
       </c>
       <c r="B268" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A269" s="1" t="s">
         <v>269</v>
       </c>
       <c r="B269" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.35">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A270" s="1" t="s">
         <v>270</v>
       </c>
       <c r="B270" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.35">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A271" s="1" t="s">
         <v>271</v>
       </c>
@@ -3910,23 +3908,23 @@
         <v>344</v>
       </c>
     </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A272" s="1" t="s">
         <v>272</v>
       </c>
       <c r="B272" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.35">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A273" s="1" t="s">
         <v>273</v>
       </c>
       <c r="B273" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A274" s="1" t="s">
         <v>274</v>
       </c>
@@ -3934,109 +3932,109 @@
         <v>359</v>
       </c>
     </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A275" s="1" t="s">
         <v>275</v>
       </c>
       <c r="B275" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.35">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A276" s="1" t="s">
         <v>276</v>
       </c>
       <c r="B276" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.35">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A277" s="1" t="s">
         <v>277</v>
       </c>
       <c r="B277" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.35">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A278" s="3" t="s">
         <v>278</v>
       </c>
       <c r="B278" s="4" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.35">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A279" s="1" t="s">
         <v>279</v>
       </c>
       <c r="B279" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.35">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A280" s="1" t="s">
         <v>280</v>
       </c>
       <c r="B280" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.35">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A281" s="1" t="s">
         <v>281</v>
       </c>
       <c r="B281" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.35">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A282" s="1" t="s">
         <v>282</v>
       </c>
       <c r="B282" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.35">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A283" s="1" t="s">
         <v>283</v>
       </c>
       <c r="B283" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.35">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A284" s="1" t="s">
         <v>284</v>
       </c>
       <c r="B284" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.35">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A285" s="3" t="s">
         <v>285</v>
       </c>
       <c r="B285" s="4"/>
     </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A286" s="1" t="s">
         <v>286</v>
       </c>
       <c r="B286" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.35">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A287" s="1" t="s">
         <v>287</v>
       </c>
       <c r="B287" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A288" s="1" t="s">
         <v>288</v>
       </c>
@@ -4044,15 +4042,15 @@
         <v>345</v>
       </c>
     </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A289" s="1" t="s">
         <v>289</v>
       </c>
       <c r="B289" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.35">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A290" s="1" t="s">
         <v>290</v>
       </c>
@@ -4060,7 +4058,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A291" s="1" t="s">
         <v>291</v>
       </c>
@@ -4068,15 +4066,15 @@
         <v>349</v>
       </c>
     </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A292" s="1" t="s">
         <v>292</v>
       </c>
       <c r="B292" t="s">
-        <v>377</v>
-      </c>
-    </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.35">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A293" s="1" t="s">
         <v>293</v>
       </c>
@@ -4084,15 +4082,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A294" s="1" t="s">
         <v>294</v>
       </c>
       <c r="B294" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A295" s="1" t="s">
         <v>295</v>
       </c>
@@ -4100,23 +4098,23 @@
         <v>337</v>
       </c>
     </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A296" s="1" t="s">
         <v>296</v>
       </c>
       <c r="B296" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.35">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A297" s="1" t="s">
         <v>297</v>
       </c>
       <c r="B297" t="s">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.35">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A298" s="1" t="s">
         <v>298</v>
       </c>
@@ -4124,15 +4122,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A299" s="1" t="s">
         <v>299</v>
       </c>
       <c r="B299" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.35">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A300" s="1" t="s">
         <v>300</v>
       </c>
@@ -4140,7 +4138,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A301" s="1" t="s">
         <v>301</v>
       </c>
@@ -4148,15 +4146,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A302" s="1" t="s">
         <v>302</v>
       </c>
       <c r="B302" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.35">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A303" s="1" t="s">
         <v>303</v>
       </c>
@@ -4164,39 +4162,39 @@
         <v>337</v>
       </c>
     </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A304" s="1" t="s">
         <v>304</v>
       </c>
       <c r="B304" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A305" s="1" t="s">
         <v>305</v>
       </c>
       <c r="B305" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.35">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A306" s="1" t="s">
         <v>306</v>
       </c>
       <c r="B306" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.35">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A307" s="1" t="s">
         <v>307</v>
       </c>
       <c r="B307" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.35">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A308" s="1" t="s">
         <v>308</v>
       </c>
@@ -4204,7 +4202,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A309" s="1" t="s">
         <v>309</v>
       </c>
@@ -4212,23 +4210,23 @@
         <v>351</v>
       </c>
     </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A310" s="1" t="s">
         <v>310</v>
       </c>
       <c r="B310" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.35">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A311" s="1" t="s">
         <v>311</v>
       </c>
       <c r="B311" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.35">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A312" s="1" t="s">
         <v>312</v>
       </c>
@@ -4236,15 +4234,15 @@
         <v>337</v>
       </c>
     </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A313" s="1" t="s">
         <v>313</v>
       </c>
       <c r="B313" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.35">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A314" s="1" t="s">
         <v>314</v>
       </c>
@@ -4252,47 +4250,47 @@
         <v>360</v>
       </c>
     </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A315" s="1" t="s">
         <v>315</v>
       </c>
       <c r="B315" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.35">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A316" s="1" t="s">
         <v>316</v>
       </c>
       <c r="B316" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.35">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A317" s="1" t="s">
         <v>317</v>
       </c>
       <c r="B317" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.35">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A318" s="1" t="s">
         <v>318</v>
       </c>
       <c r="B318" t="s">
-        <v>409</v>
-      </c>
-    </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.35">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A319" s="1" t="s">
         <v>319</v>
       </c>
       <c r="B319" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.35">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A320" s="1" t="s">
         <v>320</v>
       </c>
@@ -4300,7 +4298,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A321" s="1" t="s">
         <v>321</v>
       </c>
@@ -4308,47 +4306,47 @@
         <v>337</v>
       </c>
     </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A322" s="1" t="s">
         <v>322</v>
       </c>
       <c r="B322" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A323" s="1" t="s">
         <v>323</v>
       </c>
       <c r="B323" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A324" s="1" t="s">
         <v>324</v>
       </c>
       <c r="B324" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A325" s="1" t="s">
         <v>325</v>
       </c>
       <c r="B325" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.35">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A326" s="1" t="s">
         <v>326</v>
       </c>
       <c r="B326" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.35">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A327" s="1" t="s">
         <v>327</v>
       </c>
@@ -4356,68 +4354,68 @@
         <v>337</v>
       </c>
     </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A328" s="1" t="s">
         <v>328</v>
       </c>
       <c r="B328" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.35">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A329" s="1" t="s">
         <v>329</v>
       </c>
       <c r="B329" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.35">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A330" s="1" t="s">
         <v>330</v>
       </c>
       <c r="B330" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.35">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A331" s="1" t="s">
         <v>331</v>
       </c>
       <c r="B331" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A332" s="1" t="s">
         <v>332</v>
       </c>
       <c r="B332" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A333" s="1" t="s">
         <v>333</v>
       </c>
       <c r="B333" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="334" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A334" s="1" t="s">
         <v>334</v>
       </c>
       <c r="B334" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.35">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A335" s="1" t="s">
         <v>335</v>
       </c>
       <c r="B335" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating encounters according to tracker. Proposing kanto/national dex split in tracker
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\petrona\pokefirered-expansion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79B66B2C-232D-4A8A-8D32-A1C28108C6FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBC4399-7DBE-434C-8302-6A1B04BF53C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28890" yWindow="2800" windowWidth="9780" windowHeight="11370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$335</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="433">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="438">
   <si>
     <t>Species</t>
   </si>
@@ -1310,9 +1313,6 @@
     <t>SEAFOAM_ISLANDS_B4F</t>
   </si>
   <si>
-    <t>MT_EMBER_SUMMIT_PATH_3F</t>
-  </si>
-  <si>
     <t>ROUTE1 Water</t>
   </si>
   <si>
@@ -1335,6 +1335,24 @@
   </si>
   <si>
     <t>Roamer</t>
+  </si>
+  <si>
+    <t>POKEMON_TOWER_5F</t>
+  </si>
+  <si>
+    <t>Consider for National Dex</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Kanto Dex</t>
+  </si>
+  <si>
+    <t>Nat Dex</t>
   </si>
 </sst>
 </file>
@@ -1361,18 +1379,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1387,16 +1399,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1735,2690 +1743,3722 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
-  <dimension ref="A1:B335"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:F335"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="38" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="41.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>433</v>
+      </c>
+      <c r="E1" t="s">
+        <v>436</v>
+      </c>
+      <c r="F1" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>434</v>
+      </c>
+      <c r="E2">
+        <f>COUNTIF(C2:C335, "No")</f>
+        <v>214</v>
+      </c>
+      <c r="F2">
+        <f>COUNTIF(C2:C335, "Yes")</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B5" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B7" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B8" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B9" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B10" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B11" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B12" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B13" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B14" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B16" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B17" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B18" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B19" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B20" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B21" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B23" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B24" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B25" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B26" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B27" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B28" t="s">
         <v>348</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="C28" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C29" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B30" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C30" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B31" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C31" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B32" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C32" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B33" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C33" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B34" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C34" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B35" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C35" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B36" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C36" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B37" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B38" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C38" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B39" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C39" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B40" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C40" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B41" t="s">
         <v>358</v>
       </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C41" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B42" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B43" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B44" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C44" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B45" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C45" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B46" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B47" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C47" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B48" t="s">
         <v>362</v>
       </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C48" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B49" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C49" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B50" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" s="5" t="s">
+      <c r="C50" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B51" s="6" t="s">
+      <c r="B51" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C51" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B52" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C52" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B53" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C53" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B54" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" s="5" t="s">
+      <c r="C54" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B55" s="6" t="s">
+      <c r="B55" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C55" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B56" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C56" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B57" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B58" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C58" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B59" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B60" t="s">
         <v>366</v>
       </c>
-    </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C60" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B61" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C61" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B62" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C62" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B63" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C63" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B64" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C64" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B65" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C65" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B66" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C66" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B67" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" s="5" t="s">
+      <c r="C67" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B68" s="6" t="s">
+      <c r="B68" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C68" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B69" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C69" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B70" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C70" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B71" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C71" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B72" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C72" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B73" t="s">
         <v>371</v>
       </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C73" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B74" t="s">
         <v>372</v>
       </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C74" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B75" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C75" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B76" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C76" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B77" t="s">
         <v>374</v>
       </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C77" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B78" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C78" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B79" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C79" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B80" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C80" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B81" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C81" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>82</v>
       </c>
       <c r="B82" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B83" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C83" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B84" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B85" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C85" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B86" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B87" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" s="5" t="s">
+      <c r="C87" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A88" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B88" s="6" t="s">
+      <c r="B88" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C88" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B89" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C89" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B90" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C90" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B91" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C91" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B92" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C92" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B93" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C93" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>94</v>
       </c>
       <c r="B94" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C94" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B95" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C95" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
       <c r="B96" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C96" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>97</v>
       </c>
       <c r="B97" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C97" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B98" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C98" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B99" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C99" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>100</v>
       </c>
       <c r="B100" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C100" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>101</v>
       </c>
       <c r="B101" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C101" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B102" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C102" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B103" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C103" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>104</v>
       </c>
       <c r="B104" t="s">
         <v>354</v>
       </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C104" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B105" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C105" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>106</v>
       </c>
       <c r="B106" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C106" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B107" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C107" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B108" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C108" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B109" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" s="5" t="s">
+      <c r="C109" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A110" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B110" s="6" t="s">
+      <c r="B110" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C110" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B111" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C111" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>112</v>
       </c>
       <c r="B112" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C112" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>113</v>
       </c>
       <c r="B113" t="s">
         <v>336</v>
       </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C113" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B114" t="s">
         <v>383</v>
       </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C114" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>115</v>
       </c>
       <c r="B115" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C115" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>116</v>
       </c>
       <c r="B116" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C116" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>117</v>
       </c>
       <c r="B117" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C117" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>118</v>
       </c>
       <c r="B118" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C118" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>119</v>
       </c>
       <c r="B119" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C119" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>120</v>
       </c>
       <c r="B120" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C120" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B121" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C121" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B122" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C122" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>123</v>
       </c>
       <c r="B123" t="s">
         <v>384</v>
       </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C123" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>124</v>
       </c>
       <c r="B124" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C124" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>125</v>
       </c>
       <c r="B125" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C125" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>126</v>
       </c>
       <c r="B126" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C126" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B127" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A128" s="5" t="s">
+      <c r="C127" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A128" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="B128" s="6" t="s">
+      <c r="B128" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C128" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>129</v>
       </c>
       <c r="B129" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C129" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B130" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C130" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B131" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C131" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B132" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C132" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B133" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C133" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B134" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C134" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B135" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C135" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B136" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C136" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B137" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C137" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B138" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C138" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>139</v>
       </c>
       <c r="B139" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C139" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B140" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C140" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>141</v>
       </c>
       <c r="B141" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C141" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>142</v>
       </c>
       <c r="B142" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C142" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>143</v>
       </c>
       <c r="B143" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C143" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B144" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C144" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
       <c r="B145" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C145" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B146" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C146" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>147</v>
       </c>
       <c r="B147" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C147" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B148" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C148" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B149" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C149" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B150" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C150" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>151</v>
       </c>
       <c r="B151" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C151" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B152" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C152" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B153" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C153" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>154</v>
       </c>
       <c r="B154" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C154" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>155</v>
       </c>
       <c r="B155" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C155" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>156</v>
       </c>
       <c r="B156" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C156" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B157" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C157" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>158</v>
       </c>
       <c r="B158" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C158" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>159</v>
       </c>
       <c r="B159" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C159" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>160</v>
       </c>
       <c r="B160" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C160" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>161</v>
       </c>
       <c r="B161" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C161" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B162" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C162" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>163</v>
       </c>
       <c r="B163" t="s">
         <v>399</v>
       </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C163" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>164</v>
       </c>
       <c r="B164" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C164" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>165</v>
       </c>
       <c r="B165" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C165" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>166</v>
       </c>
       <c r="B166" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C166" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>167</v>
       </c>
       <c r="B167" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C167" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>168</v>
       </c>
       <c r="B168" t="s">
         <v>401</v>
       </c>
-    </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C168" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>169</v>
       </c>
       <c r="B169" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C169" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>170</v>
       </c>
       <c r="B170" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C170" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>171</v>
       </c>
       <c r="B171" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C171" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>172</v>
       </c>
       <c r="B172" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C172" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>173</v>
       </c>
       <c r="B173" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C173" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>174</v>
       </c>
       <c r="B174" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C174" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>175</v>
       </c>
       <c r="B175" t="s">
         <v>382</v>
       </c>
-    </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C175" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>176</v>
       </c>
       <c r="B176" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C176" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>177</v>
       </c>
       <c r="B177" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C177" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>178</v>
       </c>
       <c r="B178" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C178" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>179</v>
       </c>
       <c r="B179" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C179" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>180</v>
       </c>
       <c r="B180" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C180" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>181</v>
       </c>
       <c r="B181" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C181" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>182</v>
       </c>
       <c r="B182" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C182" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>183</v>
       </c>
       <c r="B183" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C183" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>184</v>
       </c>
       <c r="B184" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C184" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>185</v>
       </c>
       <c r="B185" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C185" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>186</v>
       </c>
       <c r="B186" t="s">
         <v>342</v>
       </c>
-    </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C186" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>187</v>
       </c>
       <c r="B187" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C187" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>188</v>
       </c>
       <c r="B188" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C188" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>189</v>
       </c>
       <c r="B189" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C189" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>190</v>
       </c>
       <c r="B190" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C190" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B191" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C191" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>192</v>
       </c>
       <c r="B192" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C192" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A193" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="B193" s="4"/>
-    </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B193" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="C193" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>194</v>
       </c>
       <c r="B194" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C194" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>195</v>
       </c>
       <c r="B195" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C195" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>196</v>
       </c>
       <c r="B196" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C196" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>197</v>
       </c>
       <c r="B197" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C197" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>198</v>
       </c>
       <c r="B198" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C198" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>199</v>
       </c>
       <c r="B199" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C199" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>200</v>
       </c>
       <c r="B200" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C200" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>201</v>
       </c>
       <c r="B201" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C201" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>202</v>
       </c>
       <c r="B202" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C202" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>203</v>
       </c>
       <c r="B203" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C203" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>204</v>
       </c>
       <c r="B204" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C204" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>205</v>
       </c>
       <c r="B205" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C205" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>206</v>
       </c>
       <c r="B206" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C206" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>207</v>
       </c>
       <c r="B207" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C207" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>208</v>
       </c>
       <c r="B208" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C208" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>209</v>
       </c>
       <c r="B209" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C209" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>210</v>
       </c>
       <c r="B210" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C210" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>211</v>
       </c>
       <c r="B211" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C211" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>212</v>
       </c>
       <c r="B212" t="s">
         <v>414</v>
       </c>
-    </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C212" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>213</v>
       </c>
       <c r="B213" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C213" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>214</v>
       </c>
       <c r="B214" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C214" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>215</v>
       </c>
       <c r="B215" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C215" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>216</v>
       </c>
       <c r="B216" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C216" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>217</v>
       </c>
       <c r="B217" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C217" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>218</v>
       </c>
       <c r="B218" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C218" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>219</v>
       </c>
       <c r="B219" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C219" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>220</v>
       </c>
       <c r="B220" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C220" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>221</v>
       </c>
       <c r="B221" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C221" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>222</v>
       </c>
       <c r="B222" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C222" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>223</v>
       </c>
       <c r="B223" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C223" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>224</v>
       </c>
       <c r="B224" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C224" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>225</v>
       </c>
       <c r="B225" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C225" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>226</v>
       </c>
       <c r="B226" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C226" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>227</v>
       </c>
       <c r="B227" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C227" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>228</v>
       </c>
       <c r="B228" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C228" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>229</v>
       </c>
       <c r="B229" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C229" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>230</v>
       </c>
       <c r="B230" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C230" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>231</v>
       </c>
       <c r="B231" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C231" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>232</v>
       </c>
       <c r="B232" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C232" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>233</v>
       </c>
       <c r="B233" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C233" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>234</v>
       </c>
       <c r="B234" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C234" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>235</v>
       </c>
       <c r="B235" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C235" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>236</v>
       </c>
       <c r="B236" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C236" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>237</v>
       </c>
       <c r="B237" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C237" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>238</v>
       </c>
       <c r="B238" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C238" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>239</v>
       </c>
       <c r="B239" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C239" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>240</v>
       </c>
       <c r="B240" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C240" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>241</v>
       </c>
       <c r="B241" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C241" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>242</v>
       </c>
       <c r="B242" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C242" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>243</v>
       </c>
       <c r="B243" t="s">
         <v>418</v>
       </c>
-    </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C243" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>244</v>
       </c>
       <c r="B244" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C244" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>245</v>
       </c>
       <c r="B245" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C245" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>246</v>
       </c>
       <c r="B246" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C246" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>247</v>
       </c>
       <c r="B247" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C247" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>248</v>
       </c>
       <c r="B248" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C248" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B249" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C249" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>250</v>
       </c>
       <c r="B250" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C250" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>251</v>
       </c>
       <c r="B251" t="s">
         <v>395</v>
       </c>
-    </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C251" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>252</v>
       </c>
       <c r="B252" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C252" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>253</v>
       </c>
       <c r="B253" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C253" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>254</v>
       </c>
       <c r="B254" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C254" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>255</v>
       </c>
       <c r="B255" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C255" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>256</v>
       </c>
       <c r="B256" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C256" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>257</v>
       </c>
       <c r="B257" t="s">
         <v>419</v>
       </c>
-    </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C257" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>258</v>
       </c>
       <c r="B258" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C258" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>259</v>
       </c>
       <c r="B259" t="s">
         <v>400</v>
       </c>
-    </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C259" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>260</v>
       </c>
       <c r="B260" t="s">
         <v>421</v>
       </c>
-    </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C260" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>261</v>
       </c>
       <c r="B261" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C261" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>262</v>
       </c>
       <c r="B262" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C262" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>263</v>
       </c>
       <c r="B263" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C263" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>264</v>
       </c>
       <c r="B264" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C264" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>265</v>
       </c>
       <c r="B265" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C265" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>266</v>
       </c>
       <c r="B266" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C266" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>267</v>
       </c>
       <c r="B267" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C267" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>268</v>
       </c>
       <c r="B268" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C268" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>269</v>
       </c>
       <c r="B269" t="s">
         <v>422</v>
       </c>
-    </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C269" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>270</v>
       </c>
       <c r="B270" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C270" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>271</v>
       </c>
       <c r="B271" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C271" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>272</v>
       </c>
       <c r="B272" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C272" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>273</v>
       </c>
       <c r="B273" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C273" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>274</v>
       </c>
       <c r="B274" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C274" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>275</v>
       </c>
       <c r="B275" t="s">
         <v>411</v>
       </c>
-    </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C275" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>276</v>
       </c>
       <c r="B276" t="s">
         <v>423</v>
       </c>
-    </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C276" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>277</v>
       </c>
       <c r="B277" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C277" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A278" s="3" t="s">
         <v>278</v>
       </c>
       <c r="B278" s="4" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+        <v>345</v>
+      </c>
+      <c r="C278" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>279</v>
       </c>
       <c r="B279" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+      <c r="C279" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>280</v>
       </c>
       <c r="B280" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+        <v>425</v>
+      </c>
+      <c r="C280" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>281</v>
       </c>
       <c r="B281" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C281" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>282</v>
       </c>
       <c r="B282" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C282" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>283</v>
       </c>
       <c r="B283" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+        <v>426</v>
+      </c>
+      <c r="C283" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>284</v>
       </c>
       <c r="B284" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+        <v>426</v>
+      </c>
+      <c r="C284" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A285" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="B285" s="4"/>
-    </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B285" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="C285" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>286</v>
       </c>
       <c r="B286" t="s">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+      <c r="C286" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>287</v>
       </c>
       <c r="B287" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C287" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>288</v>
       </c>
       <c r="B288" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C288" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>289</v>
       </c>
       <c r="B289" t="s">
         <v>405</v>
       </c>
-    </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C289" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>290</v>
       </c>
       <c r="B290" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C290" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>291</v>
       </c>
       <c r="B291" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C291" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>292</v>
       </c>
       <c r="B292" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C292" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>293</v>
       </c>
       <c r="B293" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C293" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>294</v>
       </c>
       <c r="B294" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C294" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>295</v>
       </c>
       <c r="B295" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C295" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>296</v>
       </c>
       <c r="B296" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C296" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>297</v>
       </c>
       <c r="B297" t="s">
         <v>380</v>
       </c>
-    </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C297" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>298</v>
       </c>
       <c r="B298" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C298" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>299</v>
       </c>
       <c r="B299" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C299" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>300</v>
       </c>
       <c r="B300" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="301" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C300" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>301</v>
       </c>
       <c r="B301" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="302" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C301" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>302</v>
       </c>
       <c r="B302" t="s">
         <v>373</v>
       </c>
-    </row>
-    <row r="303" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C302" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>303</v>
       </c>
       <c r="B303" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="304" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C303" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>304</v>
       </c>
       <c r="B304" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="305" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C304" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>305</v>
       </c>
       <c r="B305" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="306" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C305" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>306</v>
       </c>
       <c r="B306" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="307" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C306" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>307</v>
       </c>
       <c r="B307" t="s">
         <v>379</v>
       </c>
-    </row>
-    <row r="308" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C307" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>308</v>
       </c>
       <c r="B308" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="309" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C308" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>309</v>
       </c>
       <c r="B309" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="310" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C309" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>310</v>
       </c>
       <c r="B310" t="s">
         <v>415</v>
       </c>
-    </row>
-    <row r="311" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C310" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>311</v>
       </c>
       <c r="B311" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="312" spans="1:2" x14ac:dyDescent="0.25">
+        <v>427</v>
+      </c>
+      <c r="C311" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>312</v>
       </c>
       <c r="B312" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="313" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C312" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>313</v>
       </c>
       <c r="B313" t="s">
         <v>413</v>
       </c>
-    </row>
-    <row r="314" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C313" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="314" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>314</v>
       </c>
       <c r="B314" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="315" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C314" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>315</v>
       </c>
       <c r="B315" t="s">
         <v>417</v>
       </c>
-    </row>
-    <row r="316" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C315" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>316</v>
       </c>
       <c r="B316" t="s">
         <v>378</v>
       </c>
-    </row>
-    <row r="317" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C316" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>317</v>
       </c>
       <c r="B317" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="318" spans="1:2" x14ac:dyDescent="0.25">
+        <v>428</v>
+      </c>
+      <c r="C317" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>318</v>
       </c>
       <c r="B318" t="s">
         <v>407</v>
       </c>
-    </row>
-    <row r="319" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C318" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>319</v>
       </c>
       <c r="B319" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="320" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C319" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>320</v>
       </c>
       <c r="B320" t="s">
         <v>344</v>
       </c>
-    </row>
-    <row r="321" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C320" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>321</v>
       </c>
       <c r="B321" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="322" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C321" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>322</v>
       </c>
       <c r="B322" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="323" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C322" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>323</v>
       </c>
       <c r="B323" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="324" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C323" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>324</v>
       </c>
       <c r="B324" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="325" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C324" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="325" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>325</v>
       </c>
       <c r="B325" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="326" spans="1:2" x14ac:dyDescent="0.25">
+        <v>430</v>
+      </c>
+      <c r="C325" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="326" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>326</v>
       </c>
       <c r="B326" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="327" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C326" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="327" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>327</v>
       </c>
       <c r="B327" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="328" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C327" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="328" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>328</v>
       </c>
       <c r="B328" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="329" spans="1:2" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="C328" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="329" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>329</v>
       </c>
       <c r="B329" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="330" spans="1:2" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="C329" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="330" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>330</v>
       </c>
       <c r="B330" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="331" spans="1:2" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="C330" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="331" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>331</v>
       </c>
       <c r="B331" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="332" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C331" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="332" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>332</v>
       </c>
       <c r="B332" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="333" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C332" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="333" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>333</v>
       </c>
       <c r="B333" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="334" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C333" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="334" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>334</v>
       </c>
       <c r="B334" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="335" spans="1:2" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="C334" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="335" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>335</v>
       </c>
       <c r="B335" t="s">
-        <v>430</v>
+        <v>429</v>
+      </c>
+      <c r="C335" t="s">
+        <v>434</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C335" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="Yes"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Putting Eevee and evos back
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CBC4399-7DBE-434C-8302-6A1B04BF53C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E02C7BFB-B271-4E71-815E-2D191AA6024D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1399,21 +1399,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1743,7 +1750,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F335"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1769,7 +1775,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1781,14 +1787,14 @@
       </c>
       <c r="E2">
         <f>COUNTIF(C2:C335, "No")</f>
-        <v>214</v>
+        <v>233</v>
       </c>
       <c r="F2">
         <f>COUNTIF(C2:C335, "Yes")</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -1799,7 +1805,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -1810,7 +1816,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -1821,7 +1827,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1832,7 +1838,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -1843,7 +1849,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1854,7 +1860,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -1865,7 +1871,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1876,7 +1882,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1887,7 +1893,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -1898,7 +1904,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -1942,7 +1948,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -1953,7 +1959,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
@@ -1964,7 +1970,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
@@ -1997,7 +2003,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -2008,7 +2014,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -2019,7 +2025,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>24</v>
       </c>
@@ -2030,7 +2036,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -2041,7 +2047,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
@@ -2052,7 +2058,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -2063,7 +2069,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>28</v>
       </c>
@@ -2074,7 +2080,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>29</v>
       </c>
@@ -2085,7 +2091,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
@@ -2096,7 +2102,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
@@ -2107,7 +2113,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
@@ -2173,7 +2179,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
@@ -2184,7 +2190,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>39</v>
       </c>
@@ -2217,7 +2223,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>42</v>
       </c>
@@ -2228,7 +2234,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>43</v>
       </c>
@@ -2239,7 +2245,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>44</v>
       </c>
@@ -2250,7 +2256,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>45</v>
       </c>
@@ -2261,7 +2267,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>46</v>
       </c>
@@ -2272,7 +2278,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>47</v>
       </c>
@@ -2283,7 +2289,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
@@ -2294,7 +2300,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>49</v>
       </c>
@@ -2305,7 +2311,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>50</v>
       </c>
@@ -2382,7 +2388,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>57</v>
       </c>
@@ -2393,7 +2399,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>58</v>
       </c>
@@ -2404,7 +2410,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
@@ -2415,7 +2421,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>60</v>
       </c>
@@ -2426,7 +2432,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
@@ -2437,7 +2443,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="62" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>62</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>63</v>
       </c>
@@ -2459,7 +2465,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>64</v>
       </c>
@@ -2470,7 +2476,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -2481,7 +2487,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
@@ -2492,7 +2498,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
@@ -2503,7 +2509,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>68</v>
       </c>
@@ -2514,7 +2520,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
@@ -2525,7 +2531,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
@@ -2536,7 +2542,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
@@ -2547,7 +2553,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="72" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
@@ -2580,7 +2586,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
@@ -2591,7 +2597,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
@@ -2602,7 +2608,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
@@ -2613,7 +2619,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
@@ -2624,7 +2630,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
@@ -2635,7 +2641,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
@@ -2646,7 +2652,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
@@ -2657,7 +2663,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>82</v>
       </c>
@@ -2668,7 +2674,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
@@ -2701,7 +2707,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
@@ -2712,7 +2718,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="87" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
@@ -2811,7 +2817,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
@@ -2822,7 +2828,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>97</v>
       </c>
@@ -2833,7 +2839,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>98</v>
       </c>
@@ -2844,7 +2850,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>99</v>
       </c>
@@ -2855,7 +2861,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="100" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>100</v>
       </c>
@@ -2866,7 +2872,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>101</v>
       </c>
@@ -2874,10 +2880,10 @@
         <v>340</v>
       </c>
       <c r="C101" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>102</v>
       </c>
@@ -2885,10 +2891,10 @@
         <v>336</v>
       </c>
       <c r="C102" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>103</v>
       </c>
@@ -2896,10 +2902,10 @@
         <v>337</v>
       </c>
       <c r="C103" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>104</v>
       </c>
@@ -2910,7 +2916,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>105</v>
       </c>
@@ -2921,7 +2927,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>106</v>
       </c>
@@ -2932,7 +2938,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>107</v>
       </c>
@@ -2943,7 +2949,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>108</v>
       </c>
@@ -2954,7 +2960,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>109</v>
       </c>
@@ -2965,7 +2971,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>110</v>
       </c>
@@ -2976,7 +2982,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>111</v>
       </c>
@@ -2987,7 +2993,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="112" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>112</v>
       </c>
@@ -2998,7 +3004,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>113</v>
       </c>
@@ -3009,7 +3015,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>114</v>
       </c>
@@ -3028,7 +3034,7 @@
         <v>360</v>
       </c>
       <c r="C115" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
@@ -3039,7 +3045,7 @@
         <v>337</v>
       </c>
       <c r="C116" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
@@ -3050,7 +3056,7 @@
         <v>337</v>
       </c>
       <c r="C117" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
@@ -3061,7 +3067,7 @@
         <v>337</v>
       </c>
       <c r="C118" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
@@ -3072,7 +3078,7 @@
         <v>337</v>
       </c>
       <c r="C119" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
@@ -3083,7 +3089,7 @@
         <v>337</v>
       </c>
       <c r="C120" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
@@ -3094,7 +3100,7 @@
         <v>337</v>
       </c>
       <c r="C121" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
@@ -3105,10 +3111,10 @@
         <v>337</v>
       </c>
       <c r="C122" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>123</v>
       </c>
@@ -3119,7 +3125,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>124</v>
       </c>
@@ -3130,7 +3136,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>125</v>
       </c>
@@ -3141,7 +3147,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>126</v>
       </c>
@@ -3152,7 +3158,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="127" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>127</v>
       </c>
@@ -3163,7 +3169,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>128</v>
       </c>
@@ -3174,7 +3180,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>129</v>
       </c>
@@ -3185,7 +3191,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>130</v>
       </c>
@@ -3196,7 +3202,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>131</v>
       </c>
@@ -3207,7 +3213,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="132" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>132</v>
       </c>
@@ -3218,7 +3224,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="133" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>133</v>
       </c>
@@ -3229,7 +3235,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="134" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>134</v>
       </c>
@@ -3240,7 +3246,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>135</v>
       </c>
@@ -3251,7 +3257,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>136</v>
       </c>
@@ -3262,7 +3268,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="137" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>137</v>
       </c>
@@ -3273,7 +3279,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="138" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>138</v>
       </c>
@@ -3284,7 +3290,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="139" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>139</v>
       </c>
@@ -3295,7 +3301,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>140</v>
       </c>
@@ -3350,7 +3356,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
@@ -3361,7 +3367,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>146</v>
       </c>
@@ -3372,7 +3378,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="147" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>147</v>
       </c>
@@ -3383,7 +3389,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>148</v>
       </c>
@@ -3394,7 +3400,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="149" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>149</v>
       </c>
@@ -3405,7 +3411,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>150</v>
       </c>
@@ -3471,7 +3477,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="156" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>156</v>
       </c>
@@ -3482,7 +3488,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>157</v>
       </c>
@@ -3493,7 +3499,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="158" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>158</v>
       </c>
@@ -3504,7 +3510,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>159</v>
       </c>
@@ -3515,7 +3521,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="160" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>160</v>
       </c>
@@ -3559,7 +3565,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="164" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>164</v>
       </c>
@@ -3570,7 +3576,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>165</v>
       </c>
@@ -3581,7 +3587,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>166</v>
       </c>
@@ -3592,7 +3598,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>167</v>
       </c>
@@ -3603,7 +3609,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>168</v>
       </c>
@@ -3691,7 +3697,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>176</v>
       </c>
@@ -3702,7 +3708,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>177</v>
       </c>
@@ -3713,7 +3719,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>178</v>
       </c>
@@ -3724,7 +3730,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>179</v>
       </c>
@@ -3735,7 +3741,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>180</v>
       </c>
@@ -3746,7 +3752,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>181</v>
       </c>
@@ -3757,7 +3763,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>182</v>
       </c>
@@ -3768,7 +3774,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>183</v>
       </c>
@@ -3779,7 +3785,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="184" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>184</v>
       </c>
@@ -3790,7 +3796,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>185</v>
       </c>
@@ -3834,7 +3840,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>189</v>
       </c>
@@ -3845,7 +3851,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>190</v>
       </c>
@@ -3856,7 +3862,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="191" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>191</v>
       </c>
@@ -3867,7 +3873,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="192" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>192</v>
       </c>
@@ -3879,10 +3885,10 @@
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A193" s="3" t="s">
+      <c r="A193" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B193" s="4" t="s">
+      <c r="B193" t="s">
         <v>341</v>
       </c>
       <c r="C193" t="s">
@@ -3900,7 +3906,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="195" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>195</v>
       </c>
@@ -3908,10 +3914,10 @@
         <v>349</v>
       </c>
       <c r="C195" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>196</v>
       </c>
@@ -3919,7 +3925,7 @@
         <v>409</v>
       </c>
       <c r="C196" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.35">
@@ -3944,7 +3950,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="199" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>199</v>
       </c>
@@ -3955,7 +3961,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="200" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>200</v>
       </c>
@@ -3966,7 +3972,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="201" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>201</v>
       </c>
@@ -3977,7 +3983,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="202" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>202</v>
       </c>
@@ -3988,7 +3994,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="203" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>203</v>
       </c>
@@ -3999,7 +4005,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="204" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>204</v>
       </c>
@@ -4010,7 +4016,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="205" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>205</v>
       </c>
@@ -4021,7 +4027,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="206" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>206</v>
       </c>
@@ -4032,7 +4038,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="207" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>207</v>
       </c>
@@ -4043,7 +4049,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="208" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>208</v>
       </c>
@@ -4054,7 +4060,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="209" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>209</v>
       </c>
@@ -4065,7 +4071,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="210" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>210</v>
       </c>
@@ -4098,7 +4104,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="213" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>213</v>
       </c>
@@ -4109,7 +4115,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="214" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>214</v>
       </c>
@@ -4120,7 +4126,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="215" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>215</v>
       </c>
@@ -4131,7 +4137,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="216" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>216</v>
       </c>
@@ -4142,7 +4148,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="217" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>217</v>
       </c>
@@ -4175,7 +4181,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="220" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>220</v>
       </c>
@@ -4186,7 +4192,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="221" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>221</v>
       </c>
@@ -4197,7 +4203,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="222" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>222</v>
       </c>
@@ -4208,7 +4214,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="223" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>223</v>
       </c>
@@ -4219,7 +4225,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="224" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>224</v>
       </c>
@@ -4230,7 +4236,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="225" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>225</v>
       </c>
@@ -4241,7 +4247,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="226" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>226</v>
       </c>
@@ -4260,7 +4266,7 @@
         <v>415</v>
       </c>
       <c r="C227" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.35">
@@ -4271,7 +4277,7 @@
         <v>337</v>
       </c>
       <c r="C228" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.35">
@@ -4282,10 +4288,10 @@
         <v>337</v>
       </c>
       <c r="C229" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="230" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>230</v>
       </c>
@@ -4296,7 +4302,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="231" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>231</v>
       </c>
@@ -4307,7 +4313,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="232" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>232</v>
       </c>
@@ -4326,7 +4332,7 @@
         <v>389</v>
       </c>
       <c r="C233" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.35">
@@ -4337,7 +4343,7 @@
         <v>337</v>
       </c>
       <c r="C234" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.35">
@@ -4348,7 +4354,7 @@
         <v>337</v>
       </c>
       <c r="C235" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.35">
@@ -4359,7 +4365,7 @@
         <v>389</v>
       </c>
       <c r="C236" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.35">
@@ -4370,7 +4376,7 @@
         <v>337</v>
       </c>
       <c r="C237" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.35">
@@ -4381,7 +4387,7 @@
         <v>337</v>
       </c>
       <c r="C238" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.35">
@@ -4392,7 +4398,7 @@
         <v>389</v>
       </c>
       <c r="C239" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.35">
@@ -4403,7 +4409,7 @@
         <v>395</v>
       </c>
       <c r="C240" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.35">
@@ -4414,7 +4420,7 @@
         <v>395</v>
       </c>
       <c r="C241" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.35">
@@ -4447,7 +4453,7 @@
         <v>415</v>
       </c>
       <c r="C244" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.35">
@@ -4458,7 +4464,7 @@
         <v>395</v>
       </c>
       <c r="C245" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.35">
@@ -4469,10 +4475,10 @@
         <v>395</v>
       </c>
       <c r="C246" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="247" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>247</v>
       </c>
@@ -4483,7 +4489,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="248" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>248</v>
       </c>
@@ -4494,7 +4500,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="249" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>249</v>
       </c>
@@ -4513,7 +4519,7 @@
         <v>415</v>
       </c>
       <c r="C250" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.35">
@@ -4524,7 +4530,7 @@
         <v>395</v>
       </c>
       <c r="C251" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.35">
@@ -4535,10 +4541,10 @@
         <v>337</v>
       </c>
       <c r="C252" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="253" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>253</v>
       </c>
@@ -4549,7 +4555,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="254" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>254</v>
       </c>
@@ -4560,7 +4566,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="255" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>255</v>
       </c>
@@ -4593,7 +4599,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="258" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>258</v>
       </c>
@@ -4604,7 +4610,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="259" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>259</v>
       </c>
@@ -4615,7 +4621,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="260" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>260</v>
       </c>
@@ -4626,7 +4632,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="261" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>261</v>
       </c>
@@ -4659,7 +4665,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="264" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>264</v>
       </c>
@@ -4667,10 +4673,10 @@
         <v>350</v>
       </c>
       <c r="C264" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="265" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>265</v>
       </c>
@@ -4678,10 +4684,10 @@
         <v>389</v>
       </c>
       <c r="C265" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="266" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>266</v>
       </c>
@@ -4689,10 +4695,10 @@
         <v>357</v>
       </c>
       <c r="C266" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="267" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>267</v>
       </c>
@@ -4703,7 +4709,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="268" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>268</v>
       </c>
@@ -4714,7 +4720,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="269" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>269</v>
       </c>
@@ -4725,7 +4731,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="270" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>270</v>
       </c>
@@ -4736,7 +4742,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="271" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>271</v>
       </c>
@@ -4747,7 +4753,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="272" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>272</v>
       </c>
@@ -4780,7 +4786,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="275" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>275</v>
       </c>
@@ -4791,7 +4797,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="276" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>276</v>
       </c>
@@ -4814,10 +4820,10 @@
       </c>
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A278" s="3" t="s">
+      <c r="A278" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B278" s="4" t="s">
+      <c r="B278" t="s">
         <v>345</v>
       </c>
       <c r="C278" t="s">
@@ -4857,7 +4863,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="282" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>282</v>
       </c>
@@ -4868,7 +4874,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="283" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>283</v>
       </c>
@@ -4879,7 +4885,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="284" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>284</v>
       </c>
@@ -4890,18 +4896,18 @@
         <v>434</v>
       </c>
     </row>
-    <row r="285" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A285" s="3" t="s">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A285" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B285" s="4" t="s">
+      <c r="B285" t="s">
         <v>373</v>
       </c>
       <c r="C285" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="286" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>286</v>
       </c>
@@ -4920,7 +4926,7 @@
         <v>405</v>
       </c>
       <c r="C287" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.35">
@@ -4931,7 +4937,7 @@
         <v>345</v>
       </c>
       <c r="C288" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.35">
@@ -4942,7 +4948,7 @@
         <v>405</v>
       </c>
       <c r="C289" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.35">
@@ -4953,7 +4959,7 @@
         <v>345</v>
       </c>
       <c r="C290" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.35">
@@ -4989,7 +4995,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="294" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>294</v>
       </c>
@@ -5000,7 +5006,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="295" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>295</v>
       </c>
@@ -5011,7 +5017,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="296" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>296</v>
       </c>
@@ -5022,7 +5028,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="297" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>297</v>
       </c>
@@ -5033,7 +5039,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="298" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>298</v>
       </c>
@@ -5044,7 +5050,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="299" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>299</v>
       </c>
@@ -5055,7 +5061,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="300" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>300</v>
       </c>
@@ -5066,7 +5072,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="301" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>301</v>
       </c>
@@ -5077,7 +5083,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="302" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>302</v>
       </c>
@@ -5088,7 +5094,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="303" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>303</v>
       </c>
@@ -5121,7 +5127,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="306" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>306</v>
       </c>
@@ -5129,10 +5135,10 @@
         <v>389</v>
       </c>
       <c r="C306" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="307" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>307</v>
       </c>
@@ -5140,10 +5146,10 @@
         <v>379</v>
       </c>
       <c r="C307" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="308" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="308" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>308</v>
       </c>
@@ -5151,10 +5157,10 @@
         <v>337</v>
       </c>
       <c r="C308" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="309" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>309</v>
       </c>
@@ -5165,7 +5171,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="310" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>310</v>
       </c>
@@ -5209,7 +5215,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="314" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>314</v>
       </c>
@@ -5220,7 +5226,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="315" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>315</v>
       </c>
@@ -5264,7 +5270,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="319" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>319</v>
       </c>
@@ -5275,7 +5281,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="320" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>320</v>
       </c>
@@ -5286,7 +5292,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="321" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>321</v>
       </c>
@@ -5297,7 +5303,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="322" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>322</v>
       </c>
@@ -5308,7 +5314,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="323" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>323</v>
       </c>
@@ -5319,7 +5325,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="324" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>324</v>
       </c>
@@ -5330,7 +5336,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="325" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>325</v>
       </c>
@@ -5341,7 +5347,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="326" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>326</v>
       </c>
@@ -5352,7 +5358,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="327" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>327</v>
       </c>
@@ -5429,7 +5435,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="334" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>334</v>
       </c>
@@ -5440,7 +5446,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="335" spans="1:3" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>335</v>
       </c>
@@ -5452,13 +5458,22 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C335" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Yes"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:C335" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}"/>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Yes">
+      <formula>NOT(ISERROR(SEARCH("Yes",C1)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added skull fossil item
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89472CA6-210C-4FCD-B823-04A95F9DDA75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A99DDF-D6D9-4F95-820A-4DA20616A192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9660" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1985,7 +1985,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2035,7 +2035,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -2077,7 +2077,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>84</v>
       </c>
@@ -3295,7 +3295,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>95</v>
       </c>
@@ -3351,7 +3351,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>99</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>102</v>
       </c>
@@ -3547,7 +3547,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>113</v>
       </c>
@@ -3785,7 +3785,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130" s="1" t="s">
         <v>130</v>
       </c>
@@ -4275,7 +4275,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
         <v>165</v>
       </c>
@@ -4317,7 +4317,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A168" s="1" t="s">
         <v>168</v>
       </c>
@@ -4471,7 +4471,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A179" s="1" t="s">
         <v>179</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="183" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A183" s="1" t="s">
         <v>183</v>
       </c>
@@ -4583,7 +4583,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A187" s="1" t="s">
         <v>187</v>
       </c>
@@ -4681,7 +4681,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A194" s="1" t="s">
         <v>194</v>
       </c>
@@ -4877,7 +4877,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="208" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A208" s="1" t="s">
         <v>208</v>
       </c>
@@ -4961,7 +4961,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="214" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A214" s="1" t="s">
         <v>214</v>
       </c>
@@ -5143,7 +5143,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="227" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A227" s="1" t="s">
         <v>227</v>
       </c>
@@ -5227,7 +5227,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="233" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A233" s="1" t="s">
         <v>233</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="236" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A236" s="1" t="s">
         <v>236</v>
       </c>
@@ -5311,7 +5311,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="239" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A239" s="1" t="s">
         <v>239</v>
       </c>
@@ -5381,7 +5381,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="244" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A244" s="1" t="s">
         <v>244</v>
       </c>
@@ -5465,7 +5465,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="250" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A250" s="1" t="s">
         <v>250</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="259" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A259" s="1" t="s">
         <v>259</v>
       </c>
@@ -5675,7 +5675,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="265" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A265" s="1" t="s">
         <v>265</v>
       </c>
@@ -6249,7 +6249,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="306" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A306" s="1" t="s">
         <v>306</v>
       </c>
@@ -6305,7 +6305,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="310" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="310" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
         <v>310</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="318" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="318" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A318" s="1" t="s">
         <v>318</v>
       </c>
@@ -6691,7 +6691,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="338" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A338" s="2" t="s">
         <v>440</v>
       </c>
@@ -6702,7 +6702,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="339" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A339" s="2" t="s">
         <v>441</v>
       </c>
@@ -6713,7 +6713,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="340" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A340" s="2" t="s">
         <v>442</v>
       </c>
@@ -6724,7 +6724,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="341" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A341" s="2" t="s">
         <v>443</v>
       </c>
@@ -6735,7 +6735,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="342" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A342" s="2" t="s">
         <v>444</v>
       </c>
@@ -6746,7 +6746,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="343" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A343" s="2" t="s">
         <v>445</v>
       </c>
@@ -6768,7 +6768,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="345" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" s="2" t="s">
         <v>447</v>
       </c>
@@ -6779,7 +6779,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="346" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A346" s="2" t="s">
         <v>448</v>
       </c>
@@ -6801,7 +6801,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="348" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A348" s="2" t="s">
         <v>450</v>
       </c>
@@ -6812,7 +6812,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="349" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A349" s="2" t="s">
         <v>451</v>
       </c>
@@ -6845,7 +6845,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="352" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A352" s="2" t="s">
         <v>454</v>
       </c>
@@ -6856,7 +6856,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="353" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A353" s="2" t="s">
         <v>455</v>
       </c>
@@ -6878,7 +6878,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="355" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A355" s="2" t="s">
         <v>457</v>
       </c>
@@ -6889,7 +6889,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="356" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A356" s="2" t="s">
         <v>458</v>
       </c>
@@ -6911,7 +6911,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="358" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A358" s="2" t="s">
         <v>460</v>
       </c>
@@ -6922,7 +6922,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="359" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A359" s="2" t="s">
         <v>461</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="364" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A364" s="2" t="s">
         <v>466</v>
       </c>
@@ -6988,7 +6988,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="365" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A365" s="2" t="s">
         <v>467</v>
       </c>
@@ -6999,7 +6999,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="366" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A366" s="2" t="s">
         <v>468</v>
       </c>
@@ -7010,7 +7010,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="367" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A367" s="2" t="s">
         <v>469</v>
       </c>
@@ -7021,7 +7021,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="368" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A368" s="2" t="s">
         <v>470</v>
       </c>
@@ -7032,7 +7032,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="369" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A369" s="2" t="s">
         <v>471</v>
       </c>
@@ -7043,7 +7043,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="370" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A370" s="2" t="s">
         <v>472</v>
       </c>
@@ -7054,7 +7054,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="371" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A371" s="2" t="s">
         <v>473</v>
       </c>
@@ -7065,7 +7065,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="372" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A372" s="2" t="s">
         <v>474</v>
       </c>
@@ -7076,7 +7076,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="373" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A373" s="2" t="s">
         <v>475</v>
       </c>
@@ -7087,7 +7087,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="374" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A374" s="2" t="s">
         <v>476</v>
       </c>
@@ -7098,7 +7098,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="375" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A375" s="2" t="s">
         <v>477</v>
       </c>
@@ -7109,7 +7109,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="376" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A376" s="2" t="s">
         <v>478</v>
       </c>
@@ -7120,7 +7120,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="377" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A377" s="2" t="s">
         <v>479</v>
       </c>
@@ -7131,7 +7131,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="378" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A378" s="2" t="s">
         <v>480</v>
       </c>
@@ -7142,7 +7142,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="379" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A379" s="2" t="s">
         <v>481</v>
       </c>
@@ -7153,7 +7153,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="380" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A380" s="2" t="s">
         <v>482</v>
       </c>
@@ -7164,7 +7164,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="381" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A381" s="2" t="s">
         <v>483</v>
       </c>
@@ -7175,7 +7175,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="382" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
       <c r="A382" s="2" t="s">
         <v>484</v>
       </c>
@@ -7201,12 +7201,12 @@
   <autoFilter ref="A1:D383" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Yes"/>
+        <filter val="No"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
       <filters>
-        <filter val="Wild"/>
+        <filter val="Safari"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Update level scaling programmatically
</commit_message>
<xml_diff>
--- a/Pokedex Encounter Tracking.xlsx
+++ b/Pokedex Encounter Tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Austin\Documents\Pokemon and Gameboy\PokemonDecompBuild\pokefirered-expansion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3A99DDF-D6D9-4F95-820A-4DA20616A192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC6CA63-3D0C-4569-97C3-6B0F0FAEBA56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{7267A1CE-C028-4013-828C-44C71DAD6CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1955,7 +1955,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:F383"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2007,7 +2006,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -2021,7 +2020,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -2049,7 +2048,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -2063,7 +2062,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -2091,7 +2090,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>9</v>
       </c>
@@ -2105,7 +2104,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -2119,7 +2118,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
@@ -2133,7 +2132,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>12</v>
       </c>
@@ -2147,7 +2146,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>13</v>
       </c>
@@ -2161,7 +2160,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -2175,7 +2174,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>15</v>
       </c>
@@ -2189,7 +2188,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>16</v>
       </c>
@@ -2203,7 +2202,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>17</v>
       </c>
@@ -2217,7 +2216,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>18</v>
       </c>
@@ -2231,7 +2230,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
@@ -2245,7 +2244,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -2259,7 +2258,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>21</v>
       </c>
@@ -2273,7 +2272,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
@@ -2287,7 +2286,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>23</v>
       </c>
@@ -2301,7 +2300,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>24</v>
       </c>
@@ -2315,7 +2314,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
         <v>25</v>
       </c>
@@ -2329,7 +2328,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>26</v>
       </c>
@@ -2343,7 +2342,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
@@ -2357,7 +2356,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
         <v>28</v>
       </c>
@@ -2371,7 +2370,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>29</v>
       </c>
@@ -2385,7 +2384,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>30</v>
       </c>
@@ -2399,7 +2398,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="s">
         <v>31</v>
       </c>
@@ -2413,7 +2412,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
         <v>32</v>
       </c>
@@ -2427,7 +2426,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
         <v>33</v>
       </c>
@@ -2441,7 +2440,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>34</v>
       </c>
@@ -2455,7 +2454,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
         <v>35</v>
       </c>
@@ -2469,7 +2468,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>36</v>
       </c>
@@ -2483,7 +2482,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
         <v>37</v>
       </c>
@@ -2497,7 +2496,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
         <v>38</v>
       </c>
@@ -2511,7 +2510,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>39</v>
       </c>
@@ -2525,7 +2524,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>40</v>
       </c>
@@ -2539,7 +2538,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
         <v>41</v>
       </c>
@@ -2553,7 +2552,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
         <v>42</v>
       </c>
@@ -2567,7 +2566,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
         <v>43</v>
       </c>
@@ -2581,7 +2580,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
         <v>44</v>
       </c>
@@ -2595,7 +2594,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
         <v>45</v>
       </c>
@@ -2609,7 +2608,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
         <v>46</v>
       </c>
@@ -2623,7 +2622,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>47</v>
       </c>
@@ -2637,7 +2636,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" s="1" t="s">
         <v>48</v>
       </c>
@@ -2651,7 +2650,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>49</v>
       </c>
@@ -2665,7 +2664,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="1" t="s">
         <v>50</v>
       </c>
@@ -2679,7 +2678,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
         <v>51</v>
       </c>
@@ -2693,7 +2692,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>52</v>
       </c>
@@ -2707,7 +2706,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
@@ -2721,7 +2720,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>54</v>
       </c>
@@ -2735,7 +2734,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>55</v>
       </c>
@@ -2749,7 +2748,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>56</v>
       </c>
@@ -2763,7 +2762,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>57</v>
       </c>
@@ -2777,7 +2776,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>58</v>
       </c>
@@ -2791,7 +2790,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>59</v>
       </c>
@@ -2805,7 +2804,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>60</v>
       </c>
@@ -2819,7 +2818,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>61</v>
       </c>
@@ -2833,7 +2832,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>62</v>
       </c>
@@ -2847,7 +2846,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>63</v>
       </c>
@@ -2861,7 +2860,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>64</v>
       </c>
@@ -2875,7 +2874,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>65</v>
       </c>
@@ -2889,7 +2888,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>66</v>
       </c>
@@ -2903,7 +2902,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>67</v>
       </c>
@@ -2917,7 +2916,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>68</v>
       </c>
@@ -2931,7 +2930,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>69</v>
       </c>
@@ -2945,7 +2944,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>70</v>
       </c>
@@ -2959,7 +2958,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>71</v>
       </c>
@@ -2973,7 +2972,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>72</v>
       </c>
@@ -2987,7 +2986,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>73</v>
       </c>
@@ -3001,7 +3000,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>74</v>
       </c>
@@ -3015,7 +3014,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>75</v>
       </c>
@@ -3029,7 +3028,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>76</v>
       </c>
@@ -3043,7 +3042,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>77</v>
       </c>
@@ -3057,7 +3056,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>78</v>
       </c>
@@ -3071,7 +3070,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>79</v>
       </c>
@@ -3085,7 +3084,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>80</v>
       </c>
@@ -3099,7 +3098,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>81</v>
       </c>
@@ -3113,7 +3112,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>82</v>
       </c>
@@ -3127,7 +3126,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>83</v>
       </c>
@@ -3155,7 +3154,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>85</v>
       </c>
@@ -3169,7 +3168,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>86</v>
       </c>
@@ -3183,7 +3182,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>87</v>
       </c>
@@ -3197,7 +3196,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>88</v>
       </c>
@@ -3211,7 +3210,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>89</v>
       </c>
@@ -3225,7 +3224,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>90</v>
       </c>
@@ -3239,7 +3238,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>91</v>
       </c>
@@ -3253,7 +3252,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>92</v>
       </c>
@@ -3267,7 +3266,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>93</v>
       </c>
@@ -3281,7 +3280,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>94</v>
       </c>
@@ -3309,7 +3308,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>96</v>
       </c>
@@ -3323,7 +3322,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>97</v>
       </c>
@@ -3337,7 +3336,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>98</v>
       </c>
@@ -3365,7 +3364,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>100</v>
       </c>
@@ -3379,7 +3378,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>101</v>
       </c>
@@ -3407,7 +3406,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>103</v>
       </c>
@@ -3421,7 +3420,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>104</v>
       </c>
@@ -3435,7 +3434,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>105</v>
       </c>
@@ -3449,7 +3448,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>106</v>
       </c>
@@ -3463,7 +3462,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>107</v>
       </c>
@@ -3477,7 +3476,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>108</v>
       </c>
@@ -3491,7 +3490,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>109</v>
       </c>
@@ -3505,7 +3504,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>110</v>
       </c>
@@ -3519,7 +3518,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>111</v>
       </c>
@@ -3533,7 +3532,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>112</v>
       </c>
@@ -3561,7 +3560,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>114</v>
       </c>
@@ -3575,7 +3574,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>115</v>
       </c>
@@ -3589,7 +3588,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>116</v>
       </c>
@@ -3603,7 +3602,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>117</v>
       </c>
@@ -3617,7 +3616,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="1" t="s">
         <v>118</v>
       </c>
@@ -3631,7 +3630,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="1" t="s">
         <v>119</v>
       </c>
@@ -3645,7 +3644,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="1" t="s">
         <v>120</v>
       </c>
@@ -3659,7 +3658,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>121</v>
       </c>
@@ -3673,7 +3672,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>122</v>
       </c>
@@ -3687,7 +3686,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>123</v>
       </c>
@@ -3701,7 +3700,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="1" t="s">
         <v>124</v>
       </c>
@@ -3715,7 +3714,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125" s="1" t="s">
         <v>125</v>
       </c>
@@ -3729,7 +3728,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126" s="1" t="s">
         <v>126</v>
       </c>
@@ -3743,7 +3742,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>127</v>
       </c>
@@ -3757,7 +3756,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="1" t="s">
         <v>128</v>
       </c>
@@ -3771,7 +3770,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="129" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129" s="1" t="s">
         <v>129</v>
       </c>
@@ -3799,7 +3798,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131" s="1" t="s">
         <v>131</v>
       </c>
@@ -3813,7 +3812,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>132</v>
       </c>
@@ -3827,7 +3826,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" s="1" t="s">
         <v>133</v>
       </c>
@@ -3841,7 +3840,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="134" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" s="1" t="s">
         <v>134</v>
       </c>
@@ -3855,7 +3854,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="135" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>135</v>
       </c>
@@ -3869,7 +3868,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="136" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>136</v>
       </c>
@@ -3883,7 +3882,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="137" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>137</v>
       </c>
@@ -3897,7 +3896,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>138</v>
       </c>
@@ -3911,7 +3910,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="139" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>139</v>
       </c>
@@ -3925,7 +3924,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>140</v>
       </c>
@@ -3939,7 +3938,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>141</v>
       </c>
@@ -3953,7 +3952,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="142" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>142</v>
       </c>
@@ -3967,7 +3966,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="143" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>143</v>
       </c>
@@ -3981,7 +3980,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="144" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>144</v>
       </c>
@@ -3995,7 +3994,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" s="1" t="s">
         <v>145</v>
       </c>
@@ -4009,7 +4008,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="146" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" s="1" t="s">
         <v>146</v>
       </c>
@@ -4023,7 +4022,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="147" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" s="1" t="s">
         <v>147</v>
       </c>
@@ -4037,7 +4036,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="148" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" s="1" t="s">
         <v>148</v>
       </c>
@@ -4051,7 +4050,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="149" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A149" s="1" t="s">
         <v>149</v>
       </c>
@@ -4065,7 +4064,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="150" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A150" s="1" t="s">
         <v>150</v>
       </c>
@@ -4079,7 +4078,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="151" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A151" s="1" t="s">
         <v>151</v>
       </c>
@@ -4093,7 +4092,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="152" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A152" s="1" t="s">
         <v>152</v>
       </c>
@@ -4107,7 +4106,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="153" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>153</v>
       </c>
@@ -4121,7 +4120,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="154" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A154" s="1" t="s">
         <v>154</v>
       </c>
@@ -4135,7 +4134,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="155" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A155" s="1" t="s">
         <v>155</v>
       </c>
@@ -4149,7 +4148,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="156" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" s="1" t="s">
         <v>156</v>
       </c>
@@ -4163,7 +4162,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="157" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A157" s="1" t="s">
         <v>157</v>
       </c>
@@ -4177,7 +4176,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="158" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A158" s="1" t="s">
         <v>158</v>
       </c>
@@ -4191,7 +4190,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="159" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A159" s="1" t="s">
         <v>159</v>
       </c>
@@ -4205,7 +4204,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="160" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
         <v>160</v>
       </c>
@@ -4219,7 +4218,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
         <v>161</v>
       </c>
@@ -4233,7 +4232,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
         <v>162</v>
       </c>
@@ -4247,7 +4246,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="163" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
         <v>163</v>
       </c>
@@ -4261,7 +4260,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
         <v>164</v>
       </c>
@@ -4289,7 +4288,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
         <v>166</v>
       </c>
@@ -4303,7 +4302,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
         <v>167</v>
       </c>
@@ -4331,7 +4330,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
         <v>169</v>
       </c>
@@ -4345,7 +4344,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A170" s="1" t="s">
         <v>170</v>
       </c>
@@ -4359,7 +4358,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>171</v>
       </c>
@@ -4373,7 +4372,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A172" s="1" t="s">
         <v>172</v>
       </c>
@@ -4387,7 +4386,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A173" s="1" t="s">
         <v>173</v>
       </c>
@@ -4401,7 +4400,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A174" s="1" t="s">
         <v>174</v>
       </c>
@@ -4415,7 +4414,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A175" s="1" t="s">
         <v>175</v>
       </c>
@@ -4429,7 +4428,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A176" s="1" t="s">
         <v>176</v>
       </c>
@@ -4443,7 +4442,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A177" s="1" t="s">
         <v>177</v>
       </c>
@@ -4457,7 +4456,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>178</v>
       </c>
@@ -4485,7 +4484,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A180" s="1" t="s">
         <v>180</v>
       </c>
@@ -4499,7 +4498,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A181" s="1" t="s">
         <v>181</v>
       </c>
@@ -4513,7 +4512,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A182" s="1" t="s">
         <v>182</v>
       </c>
@@ -4541,7 +4540,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A184" s="1" t="s">
         <v>184</v>
       </c>
@@ -4555,7 +4554,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A185" s="1" t="s">
         <v>185</v>
       </c>
@@ -4569,7 +4568,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" s="1" t="s">
         <v>186</v>
       </c>
@@ -4597,7 +4596,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A188" s="1" t="s">
         <v>188</v>
       </c>
@@ -4611,7 +4610,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A189" s="1" t="s">
         <v>189</v>
       </c>
@@ -4625,7 +4624,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A190" s="1" t="s">
         <v>190</v>
       </c>
@@ -4639,7 +4638,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="191" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A191" s="1" t="s">
         <v>191</v>
       </c>
@@ -4653,7 +4652,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="192" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A192" s="1" t="s">
         <v>192</v>
       </c>
@@ -4667,7 +4666,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A193" s="1" t="s">
         <v>193</v>
       </c>
@@ -4695,7 +4694,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A195" s="1" t="s">
         <v>195</v>
       </c>
@@ -4709,7 +4708,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A196" s="1" t="s">
         <v>196</v>
       </c>
@@ -4723,7 +4722,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A197" s="1" t="s">
         <v>197</v>
       </c>
@@ -4737,7 +4736,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A198" s="1" t="s">
         <v>198</v>
       </c>
@@ -4751,7 +4750,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A199" s="1" t="s">
         <v>199</v>
       </c>
@@ -4765,7 +4764,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A200" s="1" t="s">
         <v>200</v>
       </c>
@@ -4779,7 +4778,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A201" s="1" t="s">
         <v>201</v>
       </c>
@@ -4793,7 +4792,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="202" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A202" s="1" t="s">
         <v>202</v>
       </c>
@@ -4807,7 +4806,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="203" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A203" s="1" t="s">
         <v>203</v>
       </c>
@@ -4821,7 +4820,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="204" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A204" s="1" t="s">
         <v>204</v>
       </c>
@@ -4835,7 +4834,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="205" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A205" s="1" t="s">
         <v>205</v>
       </c>
@@ -4849,7 +4848,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="206" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A206" s="1" t="s">
         <v>206</v>
       </c>
@@ -4863,7 +4862,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="207" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" s="1" t="s">
         <v>207</v>
       </c>
@@ -4891,7 +4890,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="209" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A209" s="1" t="s">
         <v>209</v>
       </c>
@@ -4905,7 +4904,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="210" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A210" s="1" t="s">
         <v>210</v>
       </c>
@@ -4919,7 +4918,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="211" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A211" s="1" t="s">
         <v>211</v>
       </c>
@@ -4933,7 +4932,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="212" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A212" s="1" t="s">
         <v>212</v>
       </c>
@@ -4947,7 +4946,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="213" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A213" s="1" t="s">
         <v>213</v>
       </c>
@@ -4975,7 +4974,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="215" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A215" s="1" t="s">
         <v>215</v>
       </c>
@@ -4989,7 +4988,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="216" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A216" s="1" t="s">
         <v>216</v>
       </c>
@@ -5003,7 +5002,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="217" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A217" s="1" t="s">
         <v>217</v>
       </c>
@@ -5017,7 +5016,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="218" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A218" s="1" t="s">
         <v>218</v>
       </c>
@@ -5031,7 +5030,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="219" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A219" s="1" t="s">
         <v>219</v>
       </c>
@@ -5045,7 +5044,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="220" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A220" s="1" t="s">
         <v>220</v>
       </c>
@@ -5059,7 +5058,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="221" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A221" s="1" t="s">
         <v>221</v>
       </c>
@@ -5073,7 +5072,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="222" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A222" s="1" t="s">
         <v>222</v>
       </c>
@@ -5087,7 +5086,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="223" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A223" s="1" t="s">
         <v>223</v>
       </c>
@@ -5101,7 +5100,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="224" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" s="1" t="s">
         <v>224</v>
       </c>
@@ -5115,7 +5114,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="225" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A225" s="1" t="s">
         <v>225</v>
       </c>
@@ -5129,7 +5128,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="226" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A226" s="1" t="s">
         <v>226</v>
       </c>
@@ -5157,7 +5156,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="228" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A228" s="1" t="s">
         <v>228</v>
       </c>
@@ -5171,7 +5170,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="229" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A229" s="1" t="s">
         <v>229</v>
       </c>
@@ -5185,7 +5184,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="230" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A230" s="1" t="s">
         <v>230</v>
       </c>
@@ -5199,7 +5198,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="231" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A231" s="1" t="s">
         <v>231</v>
       </c>
@@ -5213,7 +5212,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="232" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A232" s="1" t="s">
         <v>232</v>
       </c>
@@ -5241,7 +5240,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="234" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A234" s="1" t="s">
         <v>234</v>
       </c>
@@ -5255,7 +5254,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="235" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A235" s="1" t="s">
         <v>235</v>
       </c>
@@ -5283,7 +5282,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="237" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A237" s="1" t="s">
         <v>237</v>
       </c>
@@ -5297,7 +5296,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="238" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A238" s="1" t="s">
         <v>238</v>
       </c>
@@ -5325,7 +5324,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="240" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A240" s="1" t="s">
         <v>240</v>
       </c>
@@ -5339,7 +5338,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="241" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A241" s="1" t="s">
         <v>241</v>
       </c>
@@ -5353,7 +5352,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="242" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A242" s="1" t="s">
         <v>242</v>
       </c>
@@ -5367,7 +5366,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="243" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A243" s="1" t="s">
         <v>243</v>
       </c>
@@ -5395,7 +5394,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="245" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A245" s="1" t="s">
         <v>245</v>
       </c>
@@ -5409,7 +5408,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="246" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A246" s="1" t="s">
         <v>246</v>
       </c>
@@ -5423,7 +5422,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="247" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A247" s="1" t="s">
         <v>247</v>
       </c>
@@ -5437,7 +5436,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="248" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A248" s="1" t="s">
         <v>248</v>
       </c>
@@ -5451,7 +5450,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="249" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A249" s="1" t="s">
         <v>249</v>
       </c>
@@ -5479,7 +5478,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="251" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A251" s="1" t="s">
         <v>251</v>
       </c>
@@ -5493,7 +5492,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="252" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A252" s="1" t="s">
         <v>252</v>
       </c>
@@ -5507,7 +5506,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="253" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A253" s="1" t="s">
         <v>253</v>
       </c>
@@ -5521,7 +5520,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="254" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A254" s="1" t="s">
         <v>254</v>
       </c>
@@ -5535,7 +5534,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="255" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A255" s="1" t="s">
         <v>255</v>
       </c>
@@ -5549,7 +5548,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="256" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A256" s="1" t="s">
         <v>256</v>
       </c>
@@ -5563,7 +5562,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="257" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A257" s="1" t="s">
         <v>257</v>
       </c>
@@ -5577,7 +5576,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="258" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A258" s="1" t="s">
         <v>258</v>
       </c>
@@ -5605,7 +5604,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="260" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A260" s="1" t="s">
         <v>260</v>
       </c>
@@ -5619,7 +5618,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="261" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A261" s="1" t="s">
         <v>261</v>
       </c>
@@ -5633,7 +5632,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="262" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A262" s="1" t="s">
         <v>262</v>
       </c>
@@ -5647,7 +5646,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="263" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A263" s="1" t="s">
         <v>263</v>
       </c>
@@ -5661,7 +5660,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="264" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A264" s="1" t="s">
         <v>264</v>
       </c>
@@ -5689,7 +5688,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="266" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A266" s="1" t="s">
         <v>266</v>
       </c>
@@ -5703,7 +5702,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="267" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A267" s="1" t="s">
         <v>267</v>
       </c>
@@ -5717,7 +5716,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="268" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A268" s="1" t="s">
         <v>268</v>
       </c>
@@ -5731,7 +5730,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="269" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A269" s="1" t="s">
         <v>269</v>
       </c>
@@ -5745,7 +5744,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="270" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A270" s="1" t="s">
         <v>270</v>
       </c>
@@ -5759,7 +5758,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="271" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A271" s="1" t="s">
         <v>271</v>
       </c>
@@ -5773,7 +5772,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="272" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A272" s="1" t="s">
         <v>272</v>
       </c>
@@ -5787,7 +5786,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="273" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A273" s="1" t="s">
         <v>273</v>
       </c>
@@ -5801,7 +5800,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="274" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A274" s="1" t="s">
         <v>274</v>
       </c>
@@ -5815,7 +5814,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="275" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A275" s="1" t="s">
         <v>275</v>
       </c>
@@ -5829,7 +5828,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="276" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A276" s="1" t="s">
         <v>276</v>
       </c>
@@ -5843,7 +5842,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="277" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A277" s="1" t="s">
         <v>277</v>
       </c>
@@ -5857,7 +5856,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="278" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A278" s="1" t="s">
         <v>278</v>
       </c>
@@ -5871,7 +5870,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="279" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A279" s="1" t="s">
         <v>279</v>
       </c>
@@ -5885,7 +5884,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="280" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A280" s="1" t="s">
         <v>280</v>
       </c>
@@ -5899,7 +5898,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="281" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A281" s="1" t="s">
         <v>281</v>
       </c>
@@ -5913,7 +5912,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="282" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A282" s="1" t="s">
         <v>282</v>
       </c>
@@ -5927,7 +5926,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="283" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A283" s="1" t="s">
         <v>283</v>
       </c>
@@ -5941,7 +5940,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="284" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A284" s="1" t="s">
         <v>284</v>
       </c>
@@ -5955,7 +5954,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="285" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A285" s="1" t="s">
         <v>285</v>
       </c>
@@ -5969,7 +5968,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="286" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A286" s="1" t="s">
         <v>286</v>
       </c>
@@ -5983,7 +5982,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="287" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A287" s="1" t="s">
         <v>287</v>
       </c>
@@ -5997,7 +5996,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="288" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
         <v>288</v>
       </c>
@@ -6011,7 +6010,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="289" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A289" s="1" t="s">
         <v>289</v>
       </c>
@@ -6025,7 +6024,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="290" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A290" s="1" t="s">
         <v>290</v>
       </c>
@@ -6039,7 +6038,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="291" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A291" s="1" t="s">
         <v>291</v>
       </c>
@@ -6053,7 +6052,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="292" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A292" s="1" t="s">
         <v>292</v>
       </c>
@@ -6067,7 +6066,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="293" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A293" s="1" t="s">
         <v>293</v>
       </c>
@@ -6081,7 +6080,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="294" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A294" s="1" t="s">
         <v>294</v>
       </c>
@@ -6095,7 +6094,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="295" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A295" s="1" t="s">
         <v>295</v>
       </c>
@@ -6109,7 +6108,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="296" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A296" s="1" t="s">
         <v>296</v>
       </c>
@@ -6123,7 +6122,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="297" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A297" s="1" t="s">
         <v>297</v>
       </c>
@@ -6137,7 +6136,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="298" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A298" s="1" t="s">
         <v>298</v>
       </c>
@@ -6151,7 +6150,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="299" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A299" s="1" t="s">
         <v>299</v>
       </c>
@@ -6165,7 +6164,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="300" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A300" s="1" t="s">
         <v>300</v>
       </c>
@@ -6179,7 +6178,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="301" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A301" s="1" t="s">
         <v>301</v>
       </c>
@@ -6193,7 +6192,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="302" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A302" s="1" t="s">
         <v>302</v>
       </c>
@@ -6207,7 +6206,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="303" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A303" s="1" t="s">
         <v>303</v>
       </c>
@@ -6221,7 +6220,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="304" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A304" s="1" t="s">
         <v>304</v>
       </c>
@@ -6235,7 +6234,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="305" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A305" s="1" t="s">
         <v>305</v>
       </c>
@@ -6263,7 +6262,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="307" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A307" s="1" t="s">
         <v>307</v>
       </c>
@@ -6277,7 +6276,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="308" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A308" s="1" t="s">
         <v>308</v>
       </c>
@@ -6291,7 +6290,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="309" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="309" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A309" s="1" t="s">
         <v>309</v>
       </c>
@@ -6319,7 +6318,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="311" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="311" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A311" s="1" t="s">
         <v>311</v>
       </c>
@@ -6333,7 +6332,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="312" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="312" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A312" s="1" t="s">
         <v>312</v>
       </c>
@@ -6347,7 +6346,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="313" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="313" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A313" s="1" t="s">
         <v>313</v>
       </c>
@@ -6361,7 +6360,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="314" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="314" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A314" s="1" t="s">
         <v>314</v>
       </c>
@@ -6375,7 +6374,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="315" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="315" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A315" s="1" t="s">
         <v>315</v>
       </c>
@@ -6389,7 +6388,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="316" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="316" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A316" s="1" t="s">
         <v>316</v>
       </c>
@@ -6403,7 +6402,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="317" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A317" s="1" t="s">
         <v>317</v>
       </c>
@@ -6431,7 +6430,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="319" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="319" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A319" s="1" t="s">
         <v>319</v>
       </c>
@@ -6445,7 +6444,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="320" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A320" s="1" t="s">
         <v>320</v>
       </c>
@@ -6459,7 +6458,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="321" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A321" s="1" t="s">
         <v>321</v>
       </c>
@@ -6473,7 +6472,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="322" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="322" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
         <v>322</v>
       </c>
@@ -6487,7 +6486,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="323" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="323" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A323" s="1" t="s">
         <v>323</v>
       </c>
@@ -6501,7 +6500,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="324" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A324" s="1" t="s">
         <v>324</v>
       </c>
@@ -6515,7 +6514,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="325" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="325" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A325" s="1" t="s">
         <v>325</v>
       </c>
@@ -6529,7 +6528,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="326" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="326" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A326" s="1" t="s">
         <v>326</v>
       </c>
@@ -6543,7 +6542,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="327" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="327" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A327" s="1" t="s">
         <v>327</v>
       </c>
@@ -6557,7 +6556,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="328" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="328" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A328" s="1" t="s">
         <v>328</v>
       </c>
@@ -6571,7 +6570,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="329" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="329" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A329" s="1" t="s">
         <v>329</v>
       </c>
@@ -6585,7 +6584,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="330" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="330" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A330" s="1" t="s">
         <v>330</v>
       </c>
@@ -6599,7 +6598,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="331" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="331" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A331" s="1" t="s">
         <v>331</v>
       </c>
@@ -6613,7 +6612,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="332" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="332" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A332" s="1" t="s">
         <v>332</v>
       </c>
@@ -6627,7 +6626,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="333" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A333" s="1" t="s">
         <v>333</v>
       </c>
@@ -6641,7 +6640,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="334" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="334" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A334" s="1" t="s">
         <v>334</v>
       </c>
@@ -6655,7 +6654,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="335" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A335" s="1" t="s">
         <v>335</v>
       </c>
@@ -6669,7 +6668,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="336" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="336" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A336" s="2" t="s">
         <v>438</v>
       </c>
@@ -6680,7 +6679,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="337" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="337" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A337" s="2" t="s">
         <v>439</v>
       </c>
@@ -6691,7 +6690,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="338" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="338" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A338" s="2" t="s">
         <v>440</v>
       </c>
@@ -6702,7 +6701,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="339" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="339" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A339" s="2" t="s">
         <v>441</v>
       </c>
@@ -6713,7 +6712,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="340" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="340" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A340" s="2" t="s">
         <v>442</v>
       </c>
@@ -6724,7 +6723,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="341" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="341" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A341" s="2" t="s">
         <v>443</v>
       </c>
@@ -6735,7 +6734,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="342" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="342" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A342" s="2" t="s">
         <v>444</v>
       </c>
@@ -6746,7 +6745,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="343" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A343" s="2" t="s">
         <v>445</v>
       </c>
@@ -6757,7 +6756,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="344" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="344" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A344" s="2" t="s">
         <v>446</v>
       </c>
@@ -6768,7 +6767,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="345" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A345" s="2" t="s">
         <v>447</v>
       </c>
@@ -6779,7 +6778,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="346" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="346" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A346" s="2" t="s">
         <v>448</v>
       </c>
@@ -6790,7 +6789,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="347" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="347" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A347" s="2" t="s">
         <v>449</v>
       </c>
@@ -6801,7 +6800,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="348" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A348" s="2" t="s">
         <v>450</v>
       </c>
@@ -6812,7 +6811,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="349" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="349" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A349" s="2" t="s">
         <v>451</v>
       </c>
@@ -6823,7 +6822,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="350" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="350" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A350" s="2" t="s">
         <v>452</v>
       </c>
@@ -6834,7 +6833,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="351" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="351" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A351" s="2" t="s">
         <v>453</v>
       </c>
@@ -6845,7 +6844,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="352" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="352" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A352" s="2" t="s">
         <v>454</v>
       </c>
@@ -6856,7 +6855,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="353" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="353" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A353" s="2" t="s">
         <v>455</v>
       </c>
@@ -6867,7 +6866,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="354" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="354" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A354" s="2" t="s">
         <v>456</v>
       </c>
@@ -6878,7 +6877,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="355" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="355" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A355" s="2" t="s">
         <v>457</v>
       </c>
@@ -6889,7 +6888,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="356" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="356" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A356" s="2" t="s">
         <v>458</v>
       </c>
@@ -6900,7 +6899,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="357" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="357" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A357" s="2" t="s">
         <v>459</v>
       </c>
@@ -6911,7 +6910,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="358" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="358" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A358" s="2" t="s">
         <v>460</v>
       </c>
@@ -6922,7 +6921,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="359" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="359" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A359" s="2" t="s">
         <v>461</v>
       </c>
@@ -6933,7 +6932,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="360" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A360" s="2" t="s">
         <v>462</v>
       </c>
@@ -6944,7 +6943,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="361" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="361" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A361" s="2" t="s">
         <v>463</v>
       </c>
@@ -6955,7 +6954,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="362" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="362" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A362" s="2" t="s">
         <v>464</v>
       </c>
@@ -6966,7 +6965,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="363" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="363" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A363" s="2" t="s">
         <v>465</v>
       </c>
@@ -6977,7 +6976,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="364" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="364" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A364" s="2" t="s">
         <v>466</v>
       </c>
@@ -6988,7 +6987,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="365" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="365" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A365" s="2" t="s">
         <v>467</v>
       </c>
@@ -6999,7 +6998,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="366" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="366" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A366" s="2" t="s">
         <v>468</v>
       </c>
@@ -7010,7 +7009,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="367" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="367" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A367" s="2" t="s">
         <v>469</v>
       </c>
@@ -7021,7 +7020,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="368" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="368" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A368" s="2" t="s">
         <v>470</v>
       </c>
@@ -7032,7 +7031,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="369" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="369" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A369" s="2" t="s">
         <v>471</v>
       </c>
@@ -7043,7 +7042,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="370" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="370" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A370" s="2" t="s">
         <v>472</v>
       </c>
@@ -7054,7 +7053,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="371" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="371" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A371" s="2" t="s">
         <v>473</v>
       </c>
@@ -7065,7 +7064,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="372" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A372" s="2" t="s">
         <v>474</v>
       </c>
@@ -7076,7 +7075,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="373" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="373" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A373" s="2" t="s">
         <v>475</v>
       </c>
@@ -7087,7 +7086,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="374" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="374" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A374" s="2" t="s">
         <v>476</v>
       </c>
@@ -7098,7 +7097,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="375" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="375" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A375" s="2" t="s">
         <v>477</v>
       </c>
@@ -7109,7 +7108,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="376" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A376" s="2" t="s">
         <v>478</v>
       </c>
@@ -7120,7 +7119,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="377" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="377" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A377" s="2" t="s">
         <v>479</v>
       </c>
@@ -7131,7 +7130,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="378" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="378" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A378" s="2" t="s">
         <v>480</v>
       </c>
@@ -7142,7 +7141,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="379" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="379" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A379" s="2" t="s">
         <v>481</v>
       </c>
@@ -7153,7 +7152,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="380" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="380" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A380" s="2" t="s">
         <v>482</v>
       </c>
@@ -7164,7 +7163,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="381" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="381" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A381" s="2" t="s">
         <v>483</v>
       </c>
@@ -7175,7 +7174,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="382" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A382" s="2" t="s">
         <v>484</v>
       </c>
@@ -7186,7 +7185,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="383" spans="1:4" hidden="1" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A383" s="2" t="s">
         <v>485</v>
       </c>
@@ -7198,18 +7197,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D383" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="No"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Safari"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:D383" xr:uid="{618835FC-1E2C-432D-8A7B-662743B4A7F2}"/>
   <conditionalFormatting sqref="D2:D383">
     <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Roamer">
       <formula>NOT(ISERROR(SEARCH("Roamer",D2)))</formula>

</xml_diff>